<commit_message>
Done: change language for creating account steps
</commit_message>
<xml_diff>
--- a/language.xlsx
+++ b/language.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\OneDrive\Documents\SaigonRide_Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F74BE9B-7836-4173-BC1D-01D4BAF53E45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE3CCB65-1646-4A48-B342-9BD63B07429B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="446" uniqueCount="257">
   <si>
     <t>Project</t>
   </si>
@@ -391,9 +391,6 @@
     <t>Khám phá những góc khuất thú vị của Sài Gòn qua các lộ trình xe đạp và trải nghiệm du lịch bền vững.</t>
   </si>
   <si>
-    <t>Bạn là ai?</t>
-  </si>
-  <si>
     <t>Người dùng địa phương</t>
   </si>
   <si>
@@ -404,6 +401,396 @@
   </si>
   <si>
     <t>Khám phá dễ dàng với các tiêu chuẩn thanh toán quốc tế. Yêu cầu tải lên hộ chiếu.</t>
+  </si>
+  <si>
+    <t>Bạn là ai</t>
+  </si>
+  <si>
+    <t>EmailExists</t>
+  </si>
+  <si>
+    <t>InvalidUserType</t>
+  </si>
+  <si>
+    <t>InvalidOtp</t>
+  </si>
+  <si>
+    <t>IdentityRequired</t>
+  </si>
+  <si>
+    <t>CccdFormatError</t>
+  </si>
+  <si>
+    <t>PassportFormatError</t>
+  </si>
+  <si>
+    <t>FileRequired</t>
+  </si>
+  <si>
+    <t>FileFormatError</t>
+  </si>
+  <si>
+    <t>FileSizeError</t>
+  </si>
+  <si>
+    <t>LoginError</t>
+  </si>
+  <si>
+    <t>VerifyOtpError</t>
+  </si>
+  <si>
+    <t>OnboardingError</t>
+  </si>
+  <si>
+    <t>PendingApproval</t>
+  </si>
+  <si>
+    <t>OtpSent</t>
+  </si>
+  <si>
+    <t>PassSameError</t>
+  </si>
+  <si>
+    <t>PassMatchError</t>
+  </si>
+  <si>
+    <t>Email already exists</t>
+  </si>
+  <si>
+    <t>Invalid user type</t>
+  </si>
+  <si>
+    <t>Invalid or expired OTP</t>
+  </si>
+  <si>
+    <t>Identity number is required</t>
+  </si>
+  <si>
+    <t>CCCD must be exactly 12 digits</t>
+  </si>
+  <si>
+    <t>Passport format is invalid</t>
+  </si>
+  <si>
+    <t>File is required</t>
+  </si>
+  <si>
+    <t>Invalid file format</t>
+  </si>
+  <si>
+    <t>File too large (max 5MB)</t>
+  </si>
+  <si>
+    <t>Invalid email or password</t>
+  </si>
+  <si>
+    <t>Please verify OTP first</t>
+  </si>
+  <si>
+    <t>Please complete onboarding</t>
+  </si>
+  <si>
+    <t>Identity verification is pending approval</t>
+  </si>
+  <si>
+    <t>OTP sent successfully</t>
+  </si>
+  <si>
+    <t>New password cannot be same as old</t>
+  </si>
+  <si>
+    <t>Passwords do not match</t>
+  </si>
+  <si>
+    <t>Email này đã được đăng ký</t>
+  </si>
+  <si>
+    <t>Loại người dùng không hợp lệ</t>
+  </si>
+  <si>
+    <t>Mã OTP không đúng hoặc đã hết hạn</t>
+  </si>
+  <si>
+    <t>Vui lòng nhập số định danh (CCCD/Passport)</t>
+  </si>
+  <si>
+    <t>CCCD phải bao gồm đúng 12 chữ số</t>
+  </si>
+  <si>
+    <t>Định dạng hộ chiếu không hợp lệ</t>
+  </si>
+  <si>
+    <t>Vui lòng tải lên ảnh giấy tờ</t>
+  </si>
+  <si>
+    <t>Định dạng file không hợp lệ (chỉ nhận JPG, PNG, PDF)</t>
+  </si>
+  <si>
+    <t>File quá lớn (tối đa 5MB)</t>
+  </si>
+  <si>
+    <t>Email hoặc mật khẩu không chính xác</t>
+  </si>
+  <si>
+    <t>Vui lòng xác thực OTP trước khi đăng nhập</t>
+  </si>
+  <si>
+    <t>Vui lòng hoàn tất thông tin cơ bản</t>
+  </si>
+  <si>
+    <t>Tài khoản đang chờ quản trị viên phê duyệt giấy tờ</t>
+  </si>
+  <si>
+    <t>Mã OTP đã được gửi thành công</t>
+  </si>
+  <si>
+    <t>Mật khẩu mới không được trùng với mật khẩu cũ</t>
+  </si>
+  <si>
+    <t>Mật khẩu xác nhận không khớp</t>
+  </si>
+  <si>
+    <t>ForgotPasswordHeader</t>
+  </si>
+  <si>
+    <t>SendOtpBtn</t>
+  </si>
+  <si>
+    <t>OtpSentTo</t>
+  </si>
+  <si>
+    <t>ResetPassBtn</t>
+  </si>
+  <si>
+    <t>BackToLogin</t>
+  </si>
+  <si>
+    <t>NewPasswordPlaceholder</t>
+  </si>
+  <si>
+    <t>OtpCodePlaceholder</t>
+  </si>
+  <si>
+    <t>Forgot Password</t>
+  </si>
+  <si>
+    <t>Send OTP Code</t>
+  </si>
+  <si>
+    <t>OTP sent to:</t>
+  </si>
+  <si>
+    <t>Reset Password</t>
+  </si>
+  <si>
+    <t>Back to Login</t>
+  </si>
+  <si>
+    <t>New Password</t>
+  </si>
+  <si>
+    <t>OTP Code</t>
+  </si>
+  <si>
+    <t>Quên mật khẩu</t>
+  </si>
+  <si>
+    <t>Gửi mã OTP</t>
+  </si>
+  <si>
+    <t>Mã OTP đã được gửi đến:</t>
+  </si>
+  <si>
+    <t>Đặt lại mật khẩu</t>
+  </si>
+  <si>
+    <t>Quay lại đăng nhập</t>
+  </si>
+  <si>
+    <t>Mật khẩu mới</t>
+  </si>
+  <si>
+    <t>Mã OTP</t>
+  </si>
+  <si>
+    <t>VerifyOtpHeader</t>
+  </si>
+  <si>
+    <t>VerifyOtpSubTitle</t>
+  </si>
+  <si>
+    <t>VerifyOtpTitle</t>
+  </si>
+  <si>
+    <t>VerifyOtpDesc</t>
+  </si>
+  <si>
+    <t>SubmitBtn</t>
+  </si>
+  <si>
+    <t>TrustedPartner</t>
+  </si>
+  <si>
+    <t>GreenMobility</t>
+  </si>
+  <si>
+    <t>Email Verification</t>
+  </si>
+  <si>
+    <t>Please enter the 6-digit OTP sent to your email address</t>
+  </si>
+  <si>
+    <t>Explore the city your own way.</t>
+  </si>
+  <si>
+    <t>Just one final step to begin your journey through the streets of Saigon.</t>
+  </si>
+  <si>
+    <t>Submit</t>
+  </si>
+  <si>
+    <t>Trusted Partner</t>
+  </si>
+  <si>
+    <t>Green Mobility</t>
+  </si>
+  <si>
+    <t>Xác thực Email</t>
+  </si>
+  <si>
+    <t>Vui lòng nhập mã OTP 6 chữ số đã được gửi đến email</t>
+  </si>
+  <si>
+    <t>Khám phá thành phố theo cách của riêng bạn.</t>
+  </si>
+  <si>
+    <t>Chỉ còn một bước cuối cùng để bắt đầu hành trình trên những con phố Sài Gòn.</t>
+  </si>
+  <si>
+    <t>Xác nhận</t>
+  </si>
+  <si>
+    <t>Đối tác tin cậy</t>
+  </si>
+  <si>
+    <t>Di chuyển xanh</t>
+  </si>
+  <si>
+    <t>IdentityHeader</t>
+  </si>
+  <si>
+    <t>IdentitySubTitle</t>
+  </si>
+  <si>
+    <t>LocalIdLabel</t>
+  </si>
+  <si>
+    <t>PassportIdLabel</t>
+  </si>
+  <si>
+    <t>IdNumberPlaceholder</t>
+  </si>
+  <si>
+    <t>UploadDocLabel</t>
+  </si>
+  <si>
+    <t>UploadPrompt</t>
+  </si>
+  <si>
+    <t>SecureTitle</t>
+  </si>
+  <si>
+    <t>SecureDesc</t>
+  </si>
+  <si>
+    <t>BackBtn</t>
+  </si>
+  <si>
+    <t>Identity Verification</t>
+  </si>
+  <si>
+    <t>Please verify your identity to unlock riding access and ensure safety across the community.</t>
+  </si>
+  <si>
+    <t>CCCD Number (12 digits)</t>
+  </si>
+  <si>
+    <t>Passport Number</t>
+  </si>
+  <si>
+    <t>Enter your number...</t>
+  </si>
+  <si>
+    <t>Upload Document</t>
+  </si>
+  <si>
+    <t>Click or drag to upload photo.</t>
+  </si>
+  <si>
+    <t>Encrypted &amp; Secure</t>
+  </si>
+  <si>
+    <t>Your data is protected and used for verification only.</t>
+  </si>
+  <si>
+    <t>Back</t>
+  </si>
+  <si>
+    <t>Xác minh danh tính</t>
+  </si>
+  <si>
+    <t>Vui lòng xác minh danh tính để bắt đầu sử dụng dịch vụ và đảm bảo an toàn cho cộng đồng.</t>
+  </si>
+  <si>
+    <t>Số CCCD (12 chữ số)</t>
+  </si>
+  <si>
+    <t>Số Hộ chiếu</t>
+  </si>
+  <si>
+    <t>Nhập số của bạn...</t>
+  </si>
+  <si>
+    <t>Tải lên giấy tờ</t>
+  </si>
+  <si>
+    <t>Nhấn hoặc kéo để tải ảnh lên.</t>
+  </si>
+  <si>
+    <t>Mã hóa &amp; Bảo mật</t>
+  </si>
+  <si>
+    <t>Dữ liệu của bạn được bảo vệ và chỉ sử dụng cho mục đích xác thực.</t>
+  </si>
+  <si>
+    <t>Quay lại</t>
+  </si>
+  <si>
+    <t>RegSuccessTitle</t>
+  </si>
+  <si>
+    <t>RegSuccessDesc</t>
+  </si>
+  <si>
+    <t>StartNowBtn</t>
+  </si>
+  <si>
+    <t>Registration Successful!</t>
+  </si>
+  <si>
+    <t>Welcome to the SaigonRide community. You're now ready to start your eco-friendly journey.</t>
+  </si>
+  <si>
+    <t>Start Now</t>
+  </si>
+  <si>
+    <t>Đăng ký thành công!</t>
+  </si>
+  <si>
+    <t>Chào mừng bạn đến với cộng đồng SaigonRide. Bạn đã sẵn sàng bắt đầu hành trình xanh của mình.</t>
+  </si>
+  <si>
+    <t>Bắt đầu ngay</t>
   </si>
 </sst>
 </file>
@@ -758,7 +1145,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G43"/>
+  <dimension ref="A1:G86"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
@@ -1469,7 +1856,7 @@
         <v>116</v>
       </c>
       <c r="G39" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.3">
@@ -1486,7 +1873,7 @@
         <v>117</v>
       </c>
       <c r="G40" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.3">
@@ -1503,7 +1890,7 @@
         <v>118</v>
       </c>
       <c r="G41" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.3">
@@ -1520,7 +1907,7 @@
         <v>119</v>
       </c>
       <c r="G42" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.3">
@@ -1537,11 +1924,743 @@
         <v>120</v>
       </c>
       <c r="G43" t="s">
-        <v>127</v>
+        <v>126</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>7</v>
+      </c>
+      <c r="B44" t="s">
+        <v>8</v>
+      </c>
+      <c r="C44" t="s">
+        <v>128</v>
+      </c>
+      <c r="E44" t="s">
+        <v>144</v>
+      </c>
+      <c r="G44" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>7</v>
+      </c>
+      <c r="B45" t="s">
+        <v>8</v>
+      </c>
+      <c r="C45" t="s">
+        <v>129</v>
+      </c>
+      <c r="E45" t="s">
+        <v>145</v>
+      </c>
+      <c r="G45" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>7</v>
+      </c>
+      <c r="B46" t="s">
+        <v>8</v>
+      </c>
+      <c r="C46" t="s">
+        <v>130</v>
+      </c>
+      <c r="E46" t="s">
+        <v>146</v>
+      </c>
+      <c r="G46" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>7</v>
+      </c>
+      <c r="B47" t="s">
+        <v>8</v>
+      </c>
+      <c r="C47" t="s">
+        <v>131</v>
+      </c>
+      <c r="E47" t="s">
+        <v>147</v>
+      </c>
+      <c r="G47" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>7</v>
+      </c>
+      <c r="B48" t="s">
+        <v>8</v>
+      </c>
+      <c r="C48" t="s">
+        <v>132</v>
+      </c>
+      <c r="E48" t="s">
+        <v>148</v>
+      </c>
+      <c r="G48" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>7</v>
+      </c>
+      <c r="B49" t="s">
+        <v>8</v>
+      </c>
+      <c r="C49" t="s">
+        <v>133</v>
+      </c>
+      <c r="E49" t="s">
+        <v>149</v>
+      </c>
+      <c r="G49" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>7</v>
+      </c>
+      <c r="B50" t="s">
+        <v>8</v>
+      </c>
+      <c r="C50" t="s">
+        <v>134</v>
+      </c>
+      <c r="E50" t="s">
+        <v>150</v>
+      </c>
+      <c r="G50" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>7</v>
+      </c>
+      <c r="B51" t="s">
+        <v>8</v>
+      </c>
+      <c r="C51" t="s">
+        <v>135</v>
+      </c>
+      <c r="E51" t="s">
+        <v>151</v>
+      </c>
+      <c r="G51" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>7</v>
+      </c>
+      <c r="B52" t="s">
+        <v>8</v>
+      </c>
+      <c r="C52" t="s">
+        <v>136</v>
+      </c>
+      <c r="E52" t="s">
+        <v>152</v>
+      </c>
+      <c r="G52" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
+        <v>7</v>
+      </c>
+      <c r="B53" t="s">
+        <v>8</v>
+      </c>
+      <c r="C53" t="s">
+        <v>137</v>
+      </c>
+      <c r="E53" t="s">
+        <v>153</v>
+      </c>
+      <c r="G53" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
+        <v>7</v>
+      </c>
+      <c r="B54" t="s">
+        <v>8</v>
+      </c>
+      <c r="C54" t="s">
+        <v>138</v>
+      </c>
+      <c r="E54" t="s">
+        <v>154</v>
+      </c>
+      <c r="G54" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>7</v>
+      </c>
+      <c r="B55" t="s">
+        <v>8</v>
+      </c>
+      <c r="C55" t="s">
+        <v>139</v>
+      </c>
+      <c r="E55" t="s">
+        <v>155</v>
+      </c>
+      <c r="G55" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
+        <v>7</v>
+      </c>
+      <c r="B56" t="s">
+        <v>8</v>
+      </c>
+      <c r="C56" t="s">
+        <v>140</v>
+      </c>
+      <c r="E56" t="s">
+        <v>156</v>
+      </c>
+      <c r="G56" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
+        <v>7</v>
+      </c>
+      <c r="B57" t="s">
+        <v>8</v>
+      </c>
+      <c r="C57" t="s">
+        <v>141</v>
+      </c>
+      <c r="E57" t="s">
+        <v>157</v>
+      </c>
+      <c r="G57" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A58" t="s">
+        <v>7</v>
+      </c>
+      <c r="B58" t="s">
+        <v>8</v>
+      </c>
+      <c r="C58" t="s">
+        <v>142</v>
+      </c>
+      <c r="E58" t="s">
+        <v>158</v>
+      </c>
+      <c r="G58" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
+        <v>7</v>
+      </c>
+      <c r="B59" t="s">
+        <v>8</v>
+      </c>
+      <c r="C59" t="s">
+        <v>143</v>
+      </c>
+      <c r="E59" t="s">
+        <v>159</v>
+      </c>
+      <c r="G59" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
+        <v>7</v>
+      </c>
+      <c r="B60" t="s">
+        <v>8</v>
+      </c>
+      <c r="C60" t="s">
+        <v>176</v>
+      </c>
+      <c r="E60" t="s">
+        <v>183</v>
+      </c>
+      <c r="G60" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A61" t="s">
+        <v>7</v>
+      </c>
+      <c r="B61" t="s">
+        <v>8</v>
+      </c>
+      <c r="C61" t="s">
+        <v>177</v>
+      </c>
+      <c r="E61" t="s">
+        <v>184</v>
+      </c>
+      <c r="G61" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A62" t="s">
+        <v>7</v>
+      </c>
+      <c r="B62" t="s">
+        <v>8</v>
+      </c>
+      <c r="C62" t="s">
+        <v>178</v>
+      </c>
+      <c r="E62" t="s">
+        <v>185</v>
+      </c>
+      <c r="G62" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A63" t="s">
+        <v>7</v>
+      </c>
+      <c r="B63" t="s">
+        <v>8</v>
+      </c>
+      <c r="C63" t="s">
+        <v>179</v>
+      </c>
+      <c r="E63" t="s">
+        <v>186</v>
+      </c>
+      <c r="G63" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A64" t="s">
+        <v>7</v>
+      </c>
+      <c r="B64" t="s">
+        <v>8</v>
+      </c>
+      <c r="C64" t="s">
+        <v>180</v>
+      </c>
+      <c r="E64" t="s">
+        <v>187</v>
+      </c>
+      <c r="G64" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A65" t="s">
+        <v>7</v>
+      </c>
+      <c r="B65" t="s">
+        <v>8</v>
+      </c>
+      <c r="C65" t="s">
+        <v>181</v>
+      </c>
+      <c r="E65" t="s">
+        <v>188</v>
+      </c>
+      <c r="G65" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A66" t="s">
+        <v>7</v>
+      </c>
+      <c r="B66" t="s">
+        <v>8</v>
+      </c>
+      <c r="C66" t="s">
+        <v>182</v>
+      </c>
+      <c r="E66" t="s">
+        <v>189</v>
+      </c>
+      <c r="G66" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A67" t="s">
+        <v>7</v>
+      </c>
+      <c r="B67" t="s">
+        <v>8</v>
+      </c>
+      <c r="C67" t="s">
+        <v>197</v>
+      </c>
+      <c r="E67" t="s">
+        <v>204</v>
+      </c>
+      <c r="G67" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A68" t="s">
+        <v>7</v>
+      </c>
+      <c r="B68" t="s">
+        <v>8</v>
+      </c>
+      <c r="C68" t="s">
+        <v>198</v>
+      </c>
+      <c r="E68" t="s">
+        <v>205</v>
+      </c>
+      <c r="G68" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A69" t="s">
+        <v>7</v>
+      </c>
+      <c r="B69" t="s">
+        <v>8</v>
+      </c>
+      <c r="C69" t="s">
+        <v>199</v>
+      </c>
+      <c r="E69" t="s">
+        <v>206</v>
+      </c>
+      <c r="G69" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A70" t="s">
+        <v>7</v>
+      </c>
+      <c r="B70" t="s">
+        <v>8</v>
+      </c>
+      <c r="C70" t="s">
+        <v>200</v>
+      </c>
+      <c r="E70" t="s">
+        <v>207</v>
+      </c>
+      <c r="G70" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A71" t="s">
+        <v>7</v>
+      </c>
+      <c r="B71" t="s">
+        <v>8</v>
+      </c>
+      <c r="C71" t="s">
+        <v>201</v>
+      </c>
+      <c r="E71" t="s">
+        <v>208</v>
+      </c>
+      <c r="G71" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A72" t="s">
+        <v>7</v>
+      </c>
+      <c r="B72" t="s">
+        <v>8</v>
+      </c>
+      <c r="C72" t="s">
+        <v>202</v>
+      </c>
+      <c r="E72" t="s">
+        <v>209</v>
+      </c>
+      <c r="G72" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A73" t="s">
+        <v>7</v>
+      </c>
+      <c r="B73" t="s">
+        <v>8</v>
+      </c>
+      <c r="C73" t="s">
+        <v>203</v>
+      </c>
+      <c r="E73" t="s">
+        <v>210</v>
+      </c>
+      <c r="G73" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A74" t="s">
+        <v>7</v>
+      </c>
+      <c r="B74" t="s">
+        <v>8</v>
+      </c>
+      <c r="C74" t="s">
+        <v>218</v>
+      </c>
+      <c r="E74" t="s">
+        <v>228</v>
+      </c>
+      <c r="G74" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A75" t="s">
+        <v>7</v>
+      </c>
+      <c r="B75" t="s">
+        <v>8</v>
+      </c>
+      <c r="C75" t="s">
+        <v>219</v>
+      </c>
+      <c r="E75" t="s">
+        <v>229</v>
+      </c>
+      <c r="G75" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A76" t="s">
+        <v>7</v>
+      </c>
+      <c r="B76" t="s">
+        <v>8</v>
+      </c>
+      <c r="C76" t="s">
+        <v>220</v>
+      </c>
+      <c r="E76" t="s">
+        <v>230</v>
+      </c>
+      <c r="G76" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A77" t="s">
+        <v>7</v>
+      </c>
+      <c r="B77" t="s">
+        <v>8</v>
+      </c>
+      <c r="C77" t="s">
+        <v>221</v>
+      </c>
+      <c r="E77" t="s">
+        <v>231</v>
+      </c>
+      <c r="G77" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A78" t="s">
+        <v>7</v>
+      </c>
+      <c r="B78" t="s">
+        <v>8</v>
+      </c>
+      <c r="C78" t="s">
+        <v>222</v>
+      </c>
+      <c r="E78" t="s">
+        <v>232</v>
+      </c>
+      <c r="G78" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A79" t="s">
+        <v>7</v>
+      </c>
+      <c r="B79" t="s">
+        <v>8</v>
+      </c>
+      <c r="C79" t="s">
+        <v>223</v>
+      </c>
+      <c r="E79" t="s">
+        <v>233</v>
+      </c>
+      <c r="G79" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="80" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A80" t="s">
+        <v>7</v>
+      </c>
+      <c r="B80" t="s">
+        <v>8</v>
+      </c>
+      <c r="C80" t="s">
+        <v>224</v>
+      </c>
+      <c r="E80" t="s">
+        <v>234</v>
+      </c>
+      <c r="G80" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A81" t="s">
+        <v>7</v>
+      </c>
+      <c r="B81" t="s">
+        <v>8</v>
+      </c>
+      <c r="C81" t="s">
+        <v>225</v>
+      </c>
+      <c r="E81" t="s">
+        <v>235</v>
+      </c>
+      <c r="G81" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="82" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A82" t="s">
+        <v>7</v>
+      </c>
+      <c r="B82" t="s">
+        <v>8</v>
+      </c>
+      <c r="C82" t="s">
+        <v>226</v>
+      </c>
+      <c r="E82" t="s">
+        <v>236</v>
+      </c>
+      <c r="G82" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A83" t="s">
+        <v>7</v>
+      </c>
+      <c r="B83" t="s">
+        <v>8</v>
+      </c>
+      <c r="C83" t="s">
+        <v>227</v>
+      </c>
+      <c r="E83" t="s">
+        <v>237</v>
+      </c>
+      <c r="G83" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="84" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A84" t="s">
+        <v>7</v>
+      </c>
+      <c r="B84" t="s">
+        <v>8</v>
+      </c>
+      <c r="C84" t="s">
+        <v>248</v>
+      </c>
+      <c r="E84" t="s">
+        <v>251</v>
+      </c>
+      <c r="G84" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="85" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A85" t="s">
+        <v>7</v>
+      </c>
+      <c r="B85" t="s">
+        <v>8</v>
+      </c>
+      <c r="C85" t="s">
+        <v>249</v>
+      </c>
+      <c r="E85" t="s">
+        <v>252</v>
+      </c>
+      <c r="G85" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="86" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A86" t="s">
+        <v>7</v>
+      </c>
+      <c r="B86" t="s">
+        <v>8</v>
+      </c>
+      <c r="C86" t="s">
+        <v>250</v>
+      </c>
+      <c r="E86" t="s">
+        <v>253</v>
+      </c>
+      <c r="G86" t="s">
+        <v>256</v>
       </c>
     </row>
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1" formatColumns="0" formatRows="0" sort="0" autoFilter="0"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Done: language for station detail/lists, current
</commit_message>
<xml_diff>
--- a/language.xlsx
+++ b/language.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\OneDrive\Documents\SaigonRide_Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE3CCB65-1646-4A48-B342-9BD63B07429B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E0CAC07-BF6C-4A19-9E59-D7E6CEFFCF9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="446" uniqueCount="257">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="896" uniqueCount="520">
   <si>
     <t>Project</t>
   </si>
@@ -791,6 +791,795 @@
   </si>
   <si>
     <t>Bắt đầu ngay</t>
+  </si>
+  <si>
+    <t>Available</t>
+  </si>
+  <si>
+    <t>InUse</t>
+  </si>
+  <si>
+    <t>Maintenance</t>
+  </si>
+  <si>
+    <t>Bike</t>
+  </si>
+  <si>
+    <t>E-Scooter</t>
+  </si>
+  <si>
+    <t>Station_1_Name</t>
+  </si>
+  <si>
+    <t>District 1</t>
+  </si>
+  <si>
+    <t>In Use</t>
+  </si>
+  <si>
+    <t>Bicycle</t>
+  </si>
+  <si>
+    <t>Electric Scooter</t>
+  </si>
+  <si>
+    <t>Ben Thanh Station</t>
+  </si>
+  <si>
+    <t>Sẵn sàng</t>
+  </si>
+  <si>
+    <t>Đang sử dụng</t>
+  </si>
+  <si>
+    <t>Đang bảo trì</t>
+  </si>
+  <si>
+    <t>Xe đạp</t>
+  </si>
+  <si>
+    <t>Xe điện</t>
+  </si>
+  <si>
+    <t>Trạm Bến Thành</t>
+  </si>
+  <si>
+    <t>Quận 1</t>
+  </si>
+  <si>
+    <t>Completed</t>
+  </si>
+  <si>
+    <t>Hoàn thành</t>
+  </si>
+  <si>
+    <t>ReadyForRide</t>
+  </si>
+  <si>
+    <t>AccountLocked</t>
+  </si>
+  <si>
+    <t>ActiveAccount</t>
+  </si>
+  <si>
+    <t>BalanceLabel</t>
+  </si>
+  <si>
+    <t>QuickTopUp</t>
+  </si>
+  <si>
+    <t>AmountPlaceholder</t>
+  </si>
+  <si>
+    <t>AddFundsBtn</t>
+  </si>
+  <si>
+    <t>ExploreStations</t>
+  </si>
+  <si>
+    <t>NearbyHubs</t>
+  </si>
+  <si>
+    <t>MyLocation</t>
+  </si>
+  <si>
+    <t>StartRide</t>
+  </si>
+  <si>
+    <t>YouAreHere</t>
+  </si>
+  <si>
+    <t>CashAtStation</t>
+  </si>
+  <si>
+    <t>Ready for a ride through the city?</t>
+  </si>
+  <si>
+    <t>Account Locked</t>
+  </si>
+  <si>
+    <t>Active Account</t>
+  </si>
+  <si>
+    <t>Balance</t>
+  </si>
+  <si>
+    <t>Quick Top Up</t>
+  </si>
+  <si>
+    <t>Amount</t>
+  </si>
+  <si>
+    <t>Add Funds</t>
+  </si>
+  <si>
+    <t>Explore All Stations</t>
+  </si>
+  <si>
+    <t>Nearby Hubs</t>
+  </si>
+  <si>
+    <t>My Location</t>
+  </si>
+  <si>
+    <t>Start Ride</t>
+  </si>
+  <si>
+    <t>You are here</t>
+  </si>
+  <si>
+    <t>Cash at Station</t>
+  </si>
+  <si>
+    <t>Bạn đã sẵn sàng dạo quanh thành phố chưa?</t>
+  </si>
+  <si>
+    <t>Tài khoản bị khóa</t>
+  </si>
+  <si>
+    <t>Đang hoạt động</t>
+  </si>
+  <si>
+    <t>Số dư</t>
+  </si>
+  <si>
+    <t>Nạp tiền nhanh</t>
+  </si>
+  <si>
+    <t>Số tiền</t>
+  </si>
+  <si>
+    <t>Nạp tiền</t>
+  </si>
+  <si>
+    <t>Khám phá tất cả trạm</t>
+  </si>
+  <si>
+    <t>Trạm gần đây</t>
+  </si>
+  <si>
+    <t>Vị trí của tôi</t>
+  </si>
+  <si>
+    <t>Bắt đầu đi</t>
+  </si>
+  <si>
+    <t>Bạn ở đây</t>
+  </si>
+  <si>
+    <t>Tiền mặt tại trạm</t>
+  </si>
+  <si>
+    <t>StatusNormal</t>
+  </si>
+  <si>
+    <t>StatusAlmostEmpty</t>
+  </si>
+  <si>
+    <t>StationsNearestYou</t>
+  </si>
+  <si>
+    <t>StationsCountUnit</t>
+  </si>
+  <si>
+    <t>FullLabel</t>
+  </si>
+  <si>
+    <t>LowStockWarning</t>
+  </si>
+  <si>
+    <t>ViewStationDetail</t>
+  </si>
+  <si>
+    <t>Normal</t>
+  </si>
+  <si>
+    <t>Almost empty</t>
+  </si>
+  <si>
+    <t>Stations Nearest You</t>
+  </si>
+  <si>
+    <t>Stations</t>
+  </si>
+  <si>
+    <t>Full</t>
+  </si>
+  <si>
+    <t>LOW STOCK</t>
+  </si>
+  <si>
+    <t>View Station Detail</t>
+  </si>
+  <si>
+    <t>Bình thường</t>
+  </si>
+  <si>
+    <t>Sắp hết xe</t>
+  </si>
+  <si>
+    <t>Các trạm gần bạn nhất</t>
+  </si>
+  <si>
+    <t>Trạm</t>
+  </si>
+  <si>
+    <t>Đầy</t>
+  </si>
+  <si>
+    <t>SẮP HẾT XE</t>
+  </si>
+  <si>
+    <t>Xem chi tiết trạm</t>
+  </si>
+  <si>
+    <t>Station_2_Name</t>
+  </si>
+  <si>
+    <t>Station_3_Name</t>
+  </si>
+  <si>
+    <t>Station_4_Name</t>
+  </si>
+  <si>
+    <t>Station_5_Name</t>
+  </si>
+  <si>
+    <t>Station_6_Name</t>
+  </si>
+  <si>
+    <t>Station_7_Name</t>
+  </si>
+  <si>
+    <t>Station_8_Name</t>
+  </si>
+  <si>
+    <t>Station_9_Name</t>
+  </si>
+  <si>
+    <t>Station_10_Name</t>
+  </si>
+  <si>
+    <t>Station_11_Name</t>
+  </si>
+  <si>
+    <t>Station_12_Name</t>
+  </si>
+  <si>
+    <t>District 3 Hub</t>
+  </si>
+  <si>
+    <t>Binh Thanh Station</t>
+  </si>
+  <si>
+    <t>Thu Duc Station</t>
+  </si>
+  <si>
+    <t>Tan Binh Station</t>
+  </si>
+  <si>
+    <t>District 7 Station</t>
+  </si>
+  <si>
+    <t>Phu Nhuan Station</t>
+  </si>
+  <si>
+    <t>Go Vap Station</t>
+  </si>
+  <si>
+    <t>District 5 Station</t>
+  </si>
+  <si>
+    <t>District 10 Station</t>
+  </si>
+  <si>
+    <t>Tan Phu Station</t>
+  </si>
+  <si>
+    <t>Binh Tan Station</t>
+  </si>
+  <si>
+    <t>Trạm Quận 3</t>
+  </si>
+  <si>
+    <t>Trạm Bình Thạnh</t>
+  </si>
+  <si>
+    <t>Trạm Thủ Đức</t>
+  </si>
+  <si>
+    <t>Trạm Tân Bình</t>
+  </si>
+  <si>
+    <t>Trạm Quận 7</t>
+  </si>
+  <si>
+    <t>Trạm Phú Nhuận</t>
+  </si>
+  <si>
+    <t>Trạm Gò Vấp</t>
+  </si>
+  <si>
+    <t>Trạm Quận 5</t>
+  </si>
+  <si>
+    <t>Trạm Quận 10</t>
+  </si>
+  <si>
+    <t>Trạm Tân Phú</t>
+  </si>
+  <si>
+    <t>Trạm Bình Tân</t>
+  </si>
+  <si>
+    <t>Vo Van Tan</t>
+  </si>
+  <si>
+    <t>Dien Bien Phu</t>
+  </si>
+  <si>
+    <t>Vo Nguyen Giap</t>
+  </si>
+  <si>
+    <t>Cong Hoa</t>
+  </si>
+  <si>
+    <t>Nguyen Van Linh</t>
+  </si>
+  <si>
+    <t>Phan Xich Long</t>
+  </si>
+  <si>
+    <t>Quang Trung</t>
+  </si>
+  <si>
+    <t>Tran Hung Dao</t>
+  </si>
+  <si>
+    <t>Su Van Hanh</t>
+  </si>
+  <si>
+    <t>Lu Gia</t>
+  </si>
+  <si>
+    <t>Kinh Duong Vuong</t>
+  </si>
+  <si>
+    <t>Vo Van Tan St.</t>
+  </si>
+  <si>
+    <t>Dien Bien Phu St.</t>
+  </si>
+  <si>
+    <t>Vo Nguyen Giap St.</t>
+  </si>
+  <si>
+    <t>Cong Hoa St.</t>
+  </si>
+  <si>
+    <t>Nguyen Van Linh St.</t>
+  </si>
+  <si>
+    <t>Phan Xich Long St.</t>
+  </si>
+  <si>
+    <t>Quang Trung St.</t>
+  </si>
+  <si>
+    <t>Tran Hung Dao St.</t>
+  </si>
+  <si>
+    <t>Su Van Hanh St.</t>
+  </si>
+  <si>
+    <t>Lu Gia St.</t>
+  </si>
+  <si>
+    <t>Kinh Duong Vuong St.</t>
+  </si>
+  <si>
+    <t>Đường Võ Văn Tần.</t>
+  </si>
+  <si>
+    <t>Đường Điện Biên Phủ.</t>
+  </si>
+  <si>
+    <t>Đường Võ Nguyên Giáp.</t>
+  </si>
+  <si>
+    <t>Đường Cộng Hòa.</t>
+  </si>
+  <si>
+    <t>Đường Nguyễn Văn Linh.</t>
+  </si>
+  <si>
+    <t>Đường Phan Xích Long.</t>
+  </si>
+  <si>
+    <t>Đường Quang Trung.</t>
+  </si>
+  <si>
+    <t>Đường Trần Hưng Đạo.</t>
+  </si>
+  <si>
+    <t>Đường Sư Vạn Hạnh.</t>
+  </si>
+  <si>
+    <t>Đường Lữ Gia.</t>
+  </si>
+  <si>
+    <t>Đường Kinh Dương Vương.</t>
+  </si>
+  <si>
+    <t>BackToStationList</t>
+  </si>
+  <si>
+    <t>LowInventoryPromotion</t>
+  </si>
+  <si>
+    <t>TotalCapacity</t>
+  </si>
+  <si>
+    <t>AvailableNow</t>
+  </si>
+  <si>
+    <t>FillRate</t>
+  </si>
+  <si>
+    <t>PricingTitle</t>
+  </si>
+  <si>
+    <t>MinuteUnit</t>
+  </si>
+  <si>
+    <t>AvailableVehiclesAt</t>
+  </si>
+  <si>
+    <t>SearchIDPlaceholder</t>
+  </si>
+  <si>
+    <t>AllVehicles</t>
+  </si>
+  <si>
+    <t>FilterBtn</t>
+  </si>
+  <si>
+    <t>ThVehicleType</t>
+  </si>
+  <si>
+    <t>ThVehicleID</t>
+  </si>
+  <si>
+    <t>ThPrice</t>
+  </si>
+  <si>
+    <t>ThBattery</t>
+  </si>
+  <si>
+    <t>ThStatus</t>
+  </si>
+  <si>
+    <t>ThAction</t>
+  </si>
+  <si>
+    <t>RentNowBtn</t>
+  </si>
+  <si>
+    <t>UnavailableBtn</t>
+  </si>
+  <si>
+    <t>Back to station list</t>
+  </si>
+  <si>
+    <t>Low Inventory — Return your vehicle here for 15% discount!</t>
+  </si>
+  <si>
+    <t>Total Capacity</t>
+  </si>
+  <si>
+    <t>Available Now</t>
+  </si>
+  <si>
+    <t>Fill Rate</t>
+  </si>
+  <si>
+    <t>Pricing</t>
+  </si>
+  <si>
+    <t>minute</t>
+  </si>
+  <si>
+    <t>Available Vehicles at</t>
+  </si>
+  <si>
+    <t>Search ID...</t>
+  </si>
+  <si>
+    <t>All Vehicles</t>
+  </si>
+  <si>
+    <t>Filter</t>
+  </si>
+  <si>
+    <t>Vehicle Type</t>
+  </si>
+  <si>
+    <t>Vehicle ID</t>
+  </si>
+  <si>
+    <t>Price</t>
+  </si>
+  <si>
+    <t>Battery</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Action</t>
+  </si>
+  <si>
+    <t>Rent Now</t>
+  </si>
+  <si>
+    <t>Unavailable</t>
+  </si>
+  <si>
+    <t>Quay lại danh sách trạm</t>
+  </si>
+  <si>
+    <t>Trạm sắp hết xe — Hoàn trả xe tại đây để được giảm giá 15%!</t>
+  </si>
+  <si>
+    <t>Tổng sức chứa</t>
+  </si>
+  <si>
+    <t>Hiện có sẵn</t>
+  </si>
+  <si>
+    <t>Tỷ lệ lấp đầy</t>
+  </si>
+  <si>
+    <t>Bảng giá</t>
+  </si>
+  <si>
+    <t>phút</t>
+  </si>
+  <si>
+    <t>Các phương tiện tại</t>
+  </si>
+  <si>
+    <t>Tìm biển số...</t>
+  </si>
+  <si>
+    <t>Tất cả phương tiện</t>
+  </si>
+  <si>
+    <t>Lọc</t>
+  </si>
+  <si>
+    <t>Loại xe</t>
+  </si>
+  <si>
+    <t>Biển số</t>
+  </si>
+  <si>
+    <t>Giá thuê</t>
+  </si>
+  <si>
+    <t>Pin</t>
+  </si>
+  <si>
+    <t>Trạng thái</t>
+  </si>
+  <si>
+    <t>Hành động</t>
+  </si>
+  <si>
+    <t>Thuê ngay</t>
+  </si>
+  <si>
+    <t>Không có sẵn</t>
+  </si>
+  <si>
+    <t>RealTimeTracking</t>
+  </si>
+  <si>
+    <t>VehicleID</t>
+  </si>
+  <si>
+    <t>RideTime</t>
+  </si>
+  <si>
+    <t>Estimated</t>
+  </si>
+  <si>
+    <t>PickUp</t>
+  </si>
+  <si>
+    <t>StationTitle</t>
+  </si>
+  <si>
+    <t>TripDetails</t>
+  </si>
+  <si>
+    <t>TotalEstimated</t>
+  </si>
+  <si>
+    <t>ReturnStation</t>
+  </si>
+  <si>
+    <t>DiscountNotice</t>
+  </si>
+  <si>
+    <t>AvailableStation</t>
+  </si>
+  <si>
+    <t>FullStatus</t>
+  </si>
+  <si>
+    <t>Discount</t>
+  </si>
+  <si>
+    <t>ReturnToCaps</t>
+  </si>
+  <si>
+    <t>SelectAStation</t>
+  </si>
+  <si>
+    <t>EndRideBtn</t>
+  </si>
+  <si>
+    <t>AlertSelectStation</t>
+  </si>
+  <si>
+    <t>Theo dõi vị trí thời gian thực</t>
+  </si>
+  <si>
+    <t>Đang trong chuyến đi</t>
+  </si>
+  <si>
+    <t>Mã xe</t>
+  </si>
+  <si>
+    <t>Thời gian đi</t>
+  </si>
+  <si>
+    <t>Ước tính</t>
+  </si>
+  <si>
+    <t>Điểm lấy xe</t>
+  </si>
+  <si>
+    <t>Chi tiết chuyến đi</t>
+  </si>
+  <si>
+    <t>Tổng cộng ước tính</t>
+  </si>
+  <si>
+    <t>Trạm trả xe</t>
+  </si>
+  <si>
+    <t>Trạm đang hoạt động</t>
+  </si>
+  <si>
+    <t>đầy</t>
+  </si>
+  <si>
+    <t>giảm giá</t>
+  </si>
+  <si>
+    <t>TRẢ XE TẠI</t>
+  </si>
+  <si>
+    <t>Chọn một trạm</t>
+  </si>
+  <si>
+    <t>Kết thúc chuyến đi</t>
+  </si>
+  <si>
+    <t>Vui lòng chọn trạm trả xe trước khi kết thúc!</t>
+  </si>
+  <si>
+    <t>Real-time location tracking</t>
+  </si>
+  <si>
+    <t>Currently Renting</t>
+  </si>
+  <si>
+    <t>Ride Time</t>
+  </si>
+  <si>
+    <t>Pick-up</t>
+  </si>
+  <si>
+    <t>Station</t>
+  </si>
+  <si>
+    <t>Trip Details</t>
+  </si>
+  <si>
+    <t>Total Estimated</t>
+  </si>
+  <si>
+    <t>Return Station</t>
+  </si>
+  <si>
+    <t>Available station</t>
+  </si>
+  <si>
+    <t>full</t>
+  </si>
+  <si>
+    <t>discount</t>
+  </si>
+  <si>
+    <t>RETURN TO</t>
+  </si>
+  <si>
+    <t>Select a station</t>
+  </si>
+  <si>
+    <t>End Ride</t>
+  </si>
+  <si>
+    <t>Please select a return station first!</t>
+  </si>
+  <si>
+    <t>Returning to a low-inventory station earns you a 15% discount!</t>
+  </si>
+  <si>
+    <t>Trả xe tại trạm đang thiếu xe để nhận ưu đãi giảm giá 15%!</t>
+  </si>
+  <si>
+    <t>CurrentlyRent</t>
+  </si>
+  <si>
+    <t>PricePerMinute</t>
+  </si>
+  <si>
+    <t>Giá mỗi phút</t>
+  </si>
+  <si>
+    <t>Price per minute</t>
+  </si>
+  <si>
+    <t>StartTime</t>
+  </si>
+  <si>
+    <t>Thời gian bắt đầu</t>
+  </si>
+  <si>
+    <t>Start Time</t>
+  </si>
+  <si>
+    <t>PaymentMethod</t>
+  </si>
+  <si>
+    <t>Phương thức thanh toán</t>
+  </si>
+  <si>
+    <t>Payment Method</t>
   </si>
 </sst>
 </file>
@@ -1145,7 +1934,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G86"/>
+  <dimension ref="A1:G176"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
@@ -2656,6 +3445,1536 @@
       </c>
       <c r="G86" t="s">
         <v>256</v>
+      </c>
+    </row>
+    <row r="87" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A87" t="s">
+        <v>7</v>
+      </c>
+      <c r="B87" t="s">
+        <v>8</v>
+      </c>
+      <c r="C87" t="s">
+        <v>257</v>
+      </c>
+      <c r="E87" t="s">
+        <v>257</v>
+      </c>
+      <c r="G87" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="88" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A88" t="s">
+        <v>7</v>
+      </c>
+      <c r="B88" t="s">
+        <v>8</v>
+      </c>
+      <c r="C88" t="s">
+        <v>258</v>
+      </c>
+      <c r="E88" t="s">
+        <v>264</v>
+      </c>
+      <c r="G88" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="89" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A89" t="s">
+        <v>7</v>
+      </c>
+      <c r="B89" t="s">
+        <v>8</v>
+      </c>
+      <c r="C89" t="s">
+        <v>259</v>
+      </c>
+      <c r="E89" t="s">
+        <v>259</v>
+      </c>
+      <c r="G89" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="90" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A90" t="s">
+        <v>7</v>
+      </c>
+      <c r="B90" t="s">
+        <v>8</v>
+      </c>
+      <c r="C90" t="s">
+        <v>260</v>
+      </c>
+      <c r="E90" t="s">
+        <v>265</v>
+      </c>
+      <c r="G90" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="91" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A91" t="s">
+        <v>7</v>
+      </c>
+      <c r="B91" t="s">
+        <v>8</v>
+      </c>
+      <c r="C91" t="s">
+        <v>261</v>
+      </c>
+      <c r="E91" t="s">
+        <v>266</v>
+      </c>
+      <c r="G91" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="92" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A92" t="s">
+        <v>7</v>
+      </c>
+      <c r="B92" t="s">
+        <v>8</v>
+      </c>
+      <c r="C92" t="s">
+        <v>275</v>
+      </c>
+      <c r="E92" t="s">
+        <v>275</v>
+      </c>
+      <c r="G92" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="93" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A93" t="s">
+        <v>7</v>
+      </c>
+      <c r="B93" t="s">
+        <v>8</v>
+      </c>
+      <c r="C93" t="s">
+        <v>277</v>
+      </c>
+      <c r="E93" t="s">
+        <v>290</v>
+      </c>
+      <c r="G93" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="94" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A94" t="s">
+        <v>7</v>
+      </c>
+      <c r="B94" t="s">
+        <v>8</v>
+      </c>
+      <c r="C94" t="s">
+        <v>278</v>
+      </c>
+      <c r="E94" t="s">
+        <v>291</v>
+      </c>
+      <c r="G94" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="95" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A95" t="s">
+        <v>7</v>
+      </c>
+      <c r="B95" t="s">
+        <v>8</v>
+      </c>
+      <c r="C95" t="s">
+        <v>279</v>
+      </c>
+      <c r="E95" t="s">
+        <v>292</v>
+      </c>
+      <c r="G95" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="96" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A96" t="s">
+        <v>7</v>
+      </c>
+      <c r="B96" t="s">
+        <v>8</v>
+      </c>
+      <c r="C96" t="s">
+        <v>280</v>
+      </c>
+      <c r="E96" t="s">
+        <v>293</v>
+      </c>
+      <c r="G96" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="97" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A97" t="s">
+        <v>7</v>
+      </c>
+      <c r="B97" t="s">
+        <v>8</v>
+      </c>
+      <c r="C97" t="s">
+        <v>281</v>
+      </c>
+      <c r="E97" t="s">
+        <v>294</v>
+      </c>
+      <c r="G97" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="98" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A98" t="s">
+        <v>7</v>
+      </c>
+      <c r="B98" t="s">
+        <v>8</v>
+      </c>
+      <c r="C98" t="s">
+        <v>282</v>
+      </c>
+      <c r="E98" t="s">
+        <v>295</v>
+      </c>
+      <c r="G98" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="99" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A99" t="s">
+        <v>7</v>
+      </c>
+      <c r="B99" t="s">
+        <v>8</v>
+      </c>
+      <c r="C99" t="s">
+        <v>283</v>
+      </c>
+      <c r="E99" t="s">
+        <v>296</v>
+      </c>
+      <c r="G99" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="100" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A100" t="s">
+        <v>7</v>
+      </c>
+      <c r="B100" t="s">
+        <v>8</v>
+      </c>
+      <c r="C100" t="s">
+        <v>284</v>
+      </c>
+      <c r="E100" t="s">
+        <v>297</v>
+      </c>
+      <c r="G100" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="101" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A101" t="s">
+        <v>7</v>
+      </c>
+      <c r="B101" t="s">
+        <v>8</v>
+      </c>
+      <c r="C101" t="s">
+        <v>285</v>
+      </c>
+      <c r="E101" t="s">
+        <v>298</v>
+      </c>
+      <c r="G101" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="102" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A102" t="s">
+        <v>7</v>
+      </c>
+      <c r="B102" t="s">
+        <v>8</v>
+      </c>
+      <c r="C102" t="s">
+        <v>286</v>
+      </c>
+      <c r="E102" t="s">
+        <v>299</v>
+      </c>
+      <c r="G102" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="103" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A103" t="s">
+        <v>7</v>
+      </c>
+      <c r="B103" t="s">
+        <v>8</v>
+      </c>
+      <c r="C103" t="s">
+        <v>287</v>
+      </c>
+      <c r="E103" t="s">
+        <v>300</v>
+      </c>
+      <c r="G103" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="104" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A104" t="s">
+        <v>7</v>
+      </c>
+      <c r="B104" t="s">
+        <v>8</v>
+      </c>
+      <c r="C104" t="s">
+        <v>288</v>
+      </c>
+      <c r="E104" t="s">
+        <v>301</v>
+      </c>
+      <c r="G104" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="105" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A105" t="s">
+        <v>7</v>
+      </c>
+      <c r="B105" t="s">
+        <v>8</v>
+      </c>
+      <c r="C105" t="s">
+        <v>289</v>
+      </c>
+      <c r="E105" t="s">
+        <v>302</v>
+      </c>
+      <c r="G105" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="106" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A106" t="s">
+        <v>7</v>
+      </c>
+      <c r="B106" t="s">
+        <v>8</v>
+      </c>
+      <c r="C106" t="s">
+        <v>316</v>
+      </c>
+      <c r="E106" t="s">
+        <v>323</v>
+      </c>
+      <c r="G106" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="107" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A107" t="s">
+        <v>7</v>
+      </c>
+      <c r="B107" t="s">
+        <v>8</v>
+      </c>
+      <c r="C107" t="s">
+        <v>317</v>
+      </c>
+      <c r="E107" t="s">
+        <v>324</v>
+      </c>
+      <c r="G107" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="108" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A108" t="s">
+        <v>7</v>
+      </c>
+      <c r="B108" t="s">
+        <v>8</v>
+      </c>
+      <c r="C108" t="s">
+        <v>318</v>
+      </c>
+      <c r="E108" t="s">
+        <v>325</v>
+      </c>
+      <c r="G108" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="109" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A109" t="s">
+        <v>7</v>
+      </c>
+      <c r="B109" t="s">
+        <v>8</v>
+      </c>
+      <c r="C109" t="s">
+        <v>319</v>
+      </c>
+      <c r="E109" t="s">
+        <v>326</v>
+      </c>
+      <c r="G109" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="110" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A110" t="s">
+        <v>7</v>
+      </c>
+      <c r="B110" t="s">
+        <v>8</v>
+      </c>
+      <c r="C110" t="s">
+        <v>320</v>
+      </c>
+      <c r="E110" t="s">
+        <v>327</v>
+      </c>
+      <c r="G110" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="111" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A111" t="s">
+        <v>7</v>
+      </c>
+      <c r="B111" t="s">
+        <v>8</v>
+      </c>
+      <c r="C111" t="s">
+        <v>321</v>
+      </c>
+      <c r="E111" t="s">
+        <v>328</v>
+      </c>
+      <c r="G111" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="112" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A112" t="s">
+        <v>7</v>
+      </c>
+      <c r="B112" t="s">
+        <v>8</v>
+      </c>
+      <c r="C112" t="s">
+        <v>322</v>
+      </c>
+      <c r="E112" t="s">
+        <v>329</v>
+      </c>
+      <c r="G112" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="113" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A113" t="s">
+        <v>7</v>
+      </c>
+      <c r="B113" t="s">
+        <v>8</v>
+      </c>
+      <c r="C113" t="s">
+        <v>262</v>
+      </c>
+      <c r="E113" t="s">
+        <v>267</v>
+      </c>
+      <c r="G113" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="114" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A114" t="s">
+        <v>7</v>
+      </c>
+      <c r="B114" t="s">
+        <v>8</v>
+      </c>
+      <c r="C114" t="s">
+        <v>337</v>
+      </c>
+      <c r="E114" t="s">
+        <v>348</v>
+      </c>
+      <c r="G114" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="115" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A115" t="s">
+        <v>7</v>
+      </c>
+      <c r="B115" t="s">
+        <v>8</v>
+      </c>
+      <c r="C115" t="s">
+        <v>338</v>
+      </c>
+      <c r="E115" t="s">
+        <v>349</v>
+      </c>
+      <c r="G115" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="116" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A116" t="s">
+        <v>7</v>
+      </c>
+      <c r="B116" t="s">
+        <v>8</v>
+      </c>
+      <c r="C116" t="s">
+        <v>339</v>
+      </c>
+      <c r="E116" t="s">
+        <v>350</v>
+      </c>
+      <c r="G116" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="117" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A117" t="s">
+        <v>7</v>
+      </c>
+      <c r="B117" t="s">
+        <v>8</v>
+      </c>
+      <c r="C117" t="s">
+        <v>340</v>
+      </c>
+      <c r="E117" t="s">
+        <v>351</v>
+      </c>
+      <c r="G117" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="118" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A118" t="s">
+        <v>7</v>
+      </c>
+      <c r="B118" t="s">
+        <v>8</v>
+      </c>
+      <c r="C118" t="s">
+        <v>341</v>
+      </c>
+      <c r="E118" t="s">
+        <v>352</v>
+      </c>
+      <c r="G118" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="119" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A119" t="s">
+        <v>7</v>
+      </c>
+      <c r="B119" t="s">
+        <v>8</v>
+      </c>
+      <c r="C119" t="s">
+        <v>342</v>
+      </c>
+      <c r="E119" t="s">
+        <v>353</v>
+      </c>
+      <c r="G119" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="120" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A120" t="s">
+        <v>7</v>
+      </c>
+      <c r="B120" t="s">
+        <v>8</v>
+      </c>
+      <c r="C120" t="s">
+        <v>343</v>
+      </c>
+      <c r="E120" t="s">
+        <v>354</v>
+      </c>
+      <c r="G120" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="121" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A121" t="s">
+        <v>7</v>
+      </c>
+      <c r="B121" t="s">
+        <v>8</v>
+      </c>
+      <c r="C121" t="s">
+        <v>344</v>
+      </c>
+      <c r="E121" t="s">
+        <v>355</v>
+      </c>
+      <c r="G121" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="122" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A122" t="s">
+        <v>7</v>
+      </c>
+      <c r="B122" t="s">
+        <v>8</v>
+      </c>
+      <c r="C122" t="s">
+        <v>345</v>
+      </c>
+      <c r="E122" t="s">
+        <v>356</v>
+      </c>
+      <c r="G122" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="123" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A123" t="s">
+        <v>7</v>
+      </c>
+      <c r="B123" t="s">
+        <v>8</v>
+      </c>
+      <c r="C123" t="s">
+        <v>346</v>
+      </c>
+      <c r="E123" t="s">
+        <v>357</v>
+      </c>
+      <c r="G123" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="124" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A124" t="s">
+        <v>7</v>
+      </c>
+      <c r="B124" t="s">
+        <v>8</v>
+      </c>
+      <c r="C124" t="s">
+        <v>347</v>
+      </c>
+      <c r="E124" t="s">
+        <v>358</v>
+      </c>
+      <c r="G124" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="125" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A125" t="s">
+        <v>7</v>
+      </c>
+      <c r="B125" t="s">
+        <v>8</v>
+      </c>
+      <c r="C125" t="s">
+        <v>263</v>
+      </c>
+      <c r="E125" t="s">
+        <v>263</v>
+      </c>
+      <c r="G125" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="126" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A126" t="s">
+        <v>7</v>
+      </c>
+      <c r="B126" t="s">
+        <v>8</v>
+      </c>
+      <c r="C126" t="s">
+        <v>370</v>
+      </c>
+      <c r="E126" t="s">
+        <v>381</v>
+      </c>
+      <c r="G126" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="127" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A127" t="s">
+        <v>7</v>
+      </c>
+      <c r="B127" t="s">
+        <v>8</v>
+      </c>
+      <c r="C127" t="s">
+        <v>371</v>
+      </c>
+      <c r="E127" t="s">
+        <v>382</v>
+      </c>
+      <c r="G127" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="128" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A128" t="s">
+        <v>7</v>
+      </c>
+      <c r="B128" t="s">
+        <v>8</v>
+      </c>
+      <c r="C128" t="s">
+        <v>372</v>
+      </c>
+      <c r="E128" t="s">
+        <v>383</v>
+      </c>
+      <c r="G128" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="129" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A129" t="s">
+        <v>7</v>
+      </c>
+      <c r="B129" t="s">
+        <v>8</v>
+      </c>
+      <c r="C129" t="s">
+        <v>373</v>
+      </c>
+      <c r="E129" t="s">
+        <v>384</v>
+      </c>
+      <c r="G129" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="130" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A130" t="s">
+        <v>7</v>
+      </c>
+      <c r="B130" t="s">
+        <v>8</v>
+      </c>
+      <c r="C130" t="s">
+        <v>374</v>
+      </c>
+      <c r="E130" t="s">
+        <v>385</v>
+      </c>
+      <c r="G130" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="131" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A131" t="s">
+        <v>7</v>
+      </c>
+      <c r="B131" t="s">
+        <v>8</v>
+      </c>
+      <c r="C131" t="s">
+        <v>375</v>
+      </c>
+      <c r="E131" t="s">
+        <v>386</v>
+      </c>
+      <c r="G131" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="132" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A132" t="s">
+        <v>7</v>
+      </c>
+      <c r="B132" t="s">
+        <v>8</v>
+      </c>
+      <c r="C132" t="s">
+        <v>376</v>
+      </c>
+      <c r="E132" t="s">
+        <v>387</v>
+      </c>
+      <c r="G132" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="133" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A133" t="s">
+        <v>7</v>
+      </c>
+      <c r="B133" t="s">
+        <v>8</v>
+      </c>
+      <c r="C133" t="s">
+        <v>377</v>
+      </c>
+      <c r="E133" t="s">
+        <v>388</v>
+      </c>
+      <c r="G133" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="134" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A134" t="s">
+        <v>7</v>
+      </c>
+      <c r="B134" t="s">
+        <v>8</v>
+      </c>
+      <c r="C134" t="s">
+        <v>378</v>
+      </c>
+      <c r="E134" t="s">
+        <v>389</v>
+      </c>
+      <c r="G134" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="135" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A135" t="s">
+        <v>7</v>
+      </c>
+      <c r="B135" t="s">
+        <v>8</v>
+      </c>
+      <c r="C135" t="s">
+        <v>379</v>
+      </c>
+      <c r="E135" t="s">
+        <v>390</v>
+      </c>
+      <c r="G135" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="136" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A136" t="s">
+        <v>7</v>
+      </c>
+      <c r="B136" t="s">
+        <v>8</v>
+      </c>
+      <c r="C136" t="s">
+        <v>380</v>
+      </c>
+      <c r="E136" t="s">
+        <v>391</v>
+      </c>
+      <c r="G136" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="137" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A137" t="s">
+        <v>7</v>
+      </c>
+      <c r="B137" t="s">
+        <v>8</v>
+      </c>
+      <c r="C137" t="s">
+        <v>403</v>
+      </c>
+      <c r="E137" t="s">
+        <v>422</v>
+      </c>
+      <c r="G137" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="138" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A138" t="s">
+        <v>7</v>
+      </c>
+      <c r="B138" t="s">
+        <v>8</v>
+      </c>
+      <c r="C138" t="s">
+        <v>404</v>
+      </c>
+      <c r="E138" t="s">
+        <v>423</v>
+      </c>
+      <c r="G138" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="139" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A139" t="s">
+        <v>7</v>
+      </c>
+      <c r="B139" t="s">
+        <v>8</v>
+      </c>
+      <c r="C139" t="s">
+        <v>405</v>
+      </c>
+      <c r="E139" t="s">
+        <v>424</v>
+      </c>
+      <c r="G139" t="s">
+        <v>443</v>
+      </c>
+    </row>
+    <row r="140" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A140" t="s">
+        <v>7</v>
+      </c>
+      <c r="B140" t="s">
+        <v>8</v>
+      </c>
+      <c r="C140" t="s">
+        <v>406</v>
+      </c>
+      <c r="E140" t="s">
+        <v>425</v>
+      </c>
+      <c r="G140" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="141" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A141" t="s">
+        <v>7</v>
+      </c>
+      <c r="B141" t="s">
+        <v>8</v>
+      </c>
+      <c r="C141" t="s">
+        <v>407</v>
+      </c>
+      <c r="E141" t="s">
+        <v>426</v>
+      </c>
+      <c r="G141" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="142" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A142" t="s">
+        <v>7</v>
+      </c>
+      <c r="B142" t="s">
+        <v>8</v>
+      </c>
+      <c r="C142" t="s">
+        <v>408</v>
+      </c>
+      <c r="E142" t="s">
+        <v>427</v>
+      </c>
+      <c r="G142" t="s">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="143" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A143" t="s">
+        <v>7</v>
+      </c>
+      <c r="B143" t="s">
+        <v>8</v>
+      </c>
+      <c r="C143" t="s">
+        <v>409</v>
+      </c>
+      <c r="E143" t="s">
+        <v>428</v>
+      </c>
+      <c r="G143" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="144" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A144" t="s">
+        <v>7</v>
+      </c>
+      <c r="B144" t="s">
+        <v>8</v>
+      </c>
+      <c r="C144" t="s">
+        <v>410</v>
+      </c>
+      <c r="E144" t="s">
+        <v>429</v>
+      </c>
+      <c r="G144" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="145" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A145" t="s">
+        <v>7</v>
+      </c>
+      <c r="B145" t="s">
+        <v>8</v>
+      </c>
+      <c r="C145" t="s">
+        <v>411</v>
+      </c>
+      <c r="E145" t="s">
+        <v>430</v>
+      </c>
+      <c r="G145" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="146" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A146" t="s">
+        <v>7</v>
+      </c>
+      <c r="B146" t="s">
+        <v>8</v>
+      </c>
+      <c r="C146" t="s">
+        <v>412</v>
+      </c>
+      <c r="E146" t="s">
+        <v>431</v>
+      </c>
+      <c r="G146" t="s">
+        <v>450</v>
+      </c>
+    </row>
+    <row r="147" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A147" t="s">
+        <v>7</v>
+      </c>
+      <c r="B147" t="s">
+        <v>8</v>
+      </c>
+      <c r="C147" t="s">
+        <v>413</v>
+      </c>
+      <c r="E147" t="s">
+        <v>432</v>
+      </c>
+      <c r="G147" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="148" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A148" t="s">
+        <v>7</v>
+      </c>
+      <c r="B148" t="s">
+        <v>8</v>
+      </c>
+      <c r="C148" t="s">
+        <v>414</v>
+      </c>
+      <c r="E148" t="s">
+        <v>433</v>
+      </c>
+      <c r="G148" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="149" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A149" t="s">
+        <v>7</v>
+      </c>
+      <c r="B149" t="s">
+        <v>8</v>
+      </c>
+      <c r="C149" t="s">
+        <v>415</v>
+      </c>
+      <c r="E149" t="s">
+        <v>434</v>
+      </c>
+      <c r="G149" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="150" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A150" t="s">
+        <v>7</v>
+      </c>
+      <c r="B150" t="s">
+        <v>8</v>
+      </c>
+      <c r="C150" t="s">
+        <v>416</v>
+      </c>
+      <c r="E150" t="s">
+        <v>435</v>
+      </c>
+      <c r="G150" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="151" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A151" t="s">
+        <v>7</v>
+      </c>
+      <c r="B151" t="s">
+        <v>8</v>
+      </c>
+      <c r="C151" t="s">
+        <v>417</v>
+      </c>
+      <c r="E151" t="s">
+        <v>436</v>
+      </c>
+      <c r="G151" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="152" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A152" t="s">
+        <v>7</v>
+      </c>
+      <c r="B152" t="s">
+        <v>8</v>
+      </c>
+      <c r="C152" t="s">
+        <v>418</v>
+      </c>
+      <c r="E152" t="s">
+        <v>437</v>
+      </c>
+      <c r="G152" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="153" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A153" t="s">
+        <v>7</v>
+      </c>
+      <c r="B153" t="s">
+        <v>8</v>
+      </c>
+      <c r="C153" t="s">
+        <v>419</v>
+      </c>
+      <c r="E153" t="s">
+        <v>438</v>
+      </c>
+      <c r="G153" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="154" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A154" t="s">
+        <v>7</v>
+      </c>
+      <c r="B154" t="s">
+        <v>8</v>
+      </c>
+      <c r="C154" t="s">
+        <v>420</v>
+      </c>
+      <c r="E154" t="s">
+        <v>439</v>
+      </c>
+      <c r="G154" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="155" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A155" t="s">
+        <v>7</v>
+      </c>
+      <c r="B155" t="s">
+        <v>8</v>
+      </c>
+      <c r="C155" t="s">
+        <v>421</v>
+      </c>
+      <c r="E155" t="s">
+        <v>440</v>
+      </c>
+      <c r="G155" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="156" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A156" t="s">
+        <v>7</v>
+      </c>
+      <c r="B156" t="s">
+        <v>8</v>
+      </c>
+      <c r="C156" t="s">
+        <v>460</v>
+      </c>
+      <c r="E156" t="s">
+        <v>493</v>
+      </c>
+      <c r="G156" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="157" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A157" t="s">
+        <v>7</v>
+      </c>
+      <c r="B157" t="s">
+        <v>8</v>
+      </c>
+      <c r="C157" t="s">
+        <v>510</v>
+      </c>
+      <c r="E157" t="s">
+        <v>494</v>
+      </c>
+      <c r="G157" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="158" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A158" t="s">
+        <v>7</v>
+      </c>
+      <c r="B158" t="s">
+        <v>8</v>
+      </c>
+      <c r="C158" t="s">
+        <v>461</v>
+      </c>
+      <c r="E158" t="s">
+        <v>434</v>
+      </c>
+      <c r="G158" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="159" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A159" t="s">
+        <v>7</v>
+      </c>
+      <c r="B159" t="s">
+        <v>8</v>
+      </c>
+      <c r="C159" t="s">
+        <v>462</v>
+      </c>
+      <c r="E159" t="s">
+        <v>495</v>
+      </c>
+      <c r="G159" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="160" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A160" t="s">
+        <v>7</v>
+      </c>
+      <c r="B160" t="s">
+        <v>8</v>
+      </c>
+      <c r="C160" t="s">
+        <v>463</v>
+      </c>
+      <c r="E160" t="s">
+        <v>463</v>
+      </c>
+      <c r="G160" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="161" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A161" t="s">
+        <v>7</v>
+      </c>
+      <c r="B161" t="s">
+        <v>8</v>
+      </c>
+      <c r="C161" t="s">
+        <v>464</v>
+      </c>
+      <c r="E161" t="s">
+        <v>496</v>
+      </c>
+      <c r="G161" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="162" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A162" t="s">
+        <v>7</v>
+      </c>
+      <c r="B162" t="s">
+        <v>8</v>
+      </c>
+      <c r="C162" t="s">
+        <v>465</v>
+      </c>
+      <c r="E162" t="s">
+        <v>497</v>
+      </c>
+      <c r="G162" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="163" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A163" t="s">
+        <v>7</v>
+      </c>
+      <c r="B163" t="s">
+        <v>8</v>
+      </c>
+      <c r="C163" t="s">
+        <v>466</v>
+      </c>
+      <c r="E163" t="s">
+        <v>498</v>
+      </c>
+      <c r="G163" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="164" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A164" t="s">
+        <v>7</v>
+      </c>
+      <c r="B164" t="s">
+        <v>8</v>
+      </c>
+      <c r="C164" t="s">
+        <v>467</v>
+      </c>
+      <c r="E164" t="s">
+        <v>499</v>
+      </c>
+      <c r="G164" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="165" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A165" t="s">
+        <v>7</v>
+      </c>
+      <c r="B165" t="s">
+        <v>8</v>
+      </c>
+      <c r="C165" t="s">
+        <v>468</v>
+      </c>
+      <c r="E165" t="s">
+        <v>500</v>
+      </c>
+      <c r="G165" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="166" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A166" t="s">
+        <v>7</v>
+      </c>
+      <c r="B166" t="s">
+        <v>8</v>
+      </c>
+      <c r="C166" t="s">
+        <v>469</v>
+      </c>
+      <c r="E166" t="s">
+        <v>508</v>
+      </c>
+      <c r="G166" t="s">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="167" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A167" t="s">
+        <v>7</v>
+      </c>
+      <c r="B167" t="s">
+        <v>8</v>
+      </c>
+      <c r="C167" t="s">
+        <v>470</v>
+      </c>
+      <c r="E167" t="s">
+        <v>501</v>
+      </c>
+      <c r="G167" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="168" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A168" t="s">
+        <v>7</v>
+      </c>
+      <c r="B168" t="s">
+        <v>8</v>
+      </c>
+      <c r="C168" t="s">
+        <v>471</v>
+      </c>
+      <c r="E168" t="s">
+        <v>502</v>
+      </c>
+      <c r="G168" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="169" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A169" t="s">
+        <v>7</v>
+      </c>
+      <c r="B169" t="s">
+        <v>8</v>
+      </c>
+      <c r="C169" t="s">
+        <v>472</v>
+      </c>
+      <c r="E169" t="s">
+        <v>503</v>
+      </c>
+      <c r="G169" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="170" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A170" t="s">
+        <v>7</v>
+      </c>
+      <c r="B170" t="s">
+        <v>8</v>
+      </c>
+      <c r="C170" t="s">
+        <v>473</v>
+      </c>
+      <c r="E170" t="s">
+        <v>504</v>
+      </c>
+      <c r="G170" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="171" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A171" t="s">
+        <v>7</v>
+      </c>
+      <c r="B171" t="s">
+        <v>8</v>
+      </c>
+      <c r="C171" t="s">
+        <v>474</v>
+      </c>
+      <c r="E171" t="s">
+        <v>505</v>
+      </c>
+      <c r="G171" t="s">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="172" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A172" t="s">
+        <v>7</v>
+      </c>
+      <c r="B172" t="s">
+        <v>8</v>
+      </c>
+      <c r="C172" t="s">
+        <v>475</v>
+      </c>
+      <c r="E172" t="s">
+        <v>506</v>
+      </c>
+      <c r="G172" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="173" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A173" t="s">
+        <v>7</v>
+      </c>
+      <c r="B173" t="s">
+        <v>8</v>
+      </c>
+      <c r="C173" t="s">
+        <v>476</v>
+      </c>
+      <c r="E173" t="s">
+        <v>507</v>
+      </c>
+      <c r="G173" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="174" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A174" t="s">
+        <v>7</v>
+      </c>
+      <c r="B174" t="s">
+        <v>8</v>
+      </c>
+      <c r="C174" t="s">
+        <v>511</v>
+      </c>
+      <c r="E174" t="s">
+        <v>513</v>
+      </c>
+      <c r="G174" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="175" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A175" t="s">
+        <v>7</v>
+      </c>
+      <c r="B175" t="s">
+        <v>8</v>
+      </c>
+      <c r="C175" t="s">
+        <v>514</v>
+      </c>
+      <c r="E175" t="s">
+        <v>516</v>
+      </c>
+      <c r="G175" t="s">
+        <v>515</v>
+      </c>
+    </row>
+    <row r="176" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A176" t="s">
+        <v>7</v>
+      </c>
+      <c r="B176" t="s">
+        <v>8</v>
+      </c>
+      <c r="C176" t="s">
+        <v>517</v>
+      </c>
+      <c r="E176" t="s">
+        <v>519</v>
+      </c>
+      <c r="G176" t="s">
+        <v>518</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Done bill, payment success, fix current
</commit_message>
<xml_diff>
--- a/language.xlsx
+++ b/language.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\OneDrive\Documents\SaigonRide_Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E0CAC07-BF6C-4A19-9E59-D7E6CEFFCF9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F639CE3-17BA-4DA7-86C0-8BD7C3C4544F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="896" uniqueCount="520">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1041" uniqueCount="605">
   <si>
     <t>Project</t>
   </si>
@@ -1393,9 +1393,6 @@
     <t>Trạng thái</t>
   </si>
   <si>
-    <t>Hành động</t>
-  </si>
-  <si>
     <t>Thuê ngay</t>
   </si>
   <si>
@@ -1474,9 +1471,6 @@
     <t>Chi tiết chuyến đi</t>
   </si>
   <si>
-    <t>Tổng cộng ước tính</t>
-  </si>
-  <si>
     <t>Trạm trả xe</t>
   </si>
   <si>
@@ -1580,6 +1574,267 @@
   </si>
   <si>
     <t>Payment Method</t>
+  </si>
+  <si>
+    <t>Vehicle</t>
+  </si>
+  <si>
+    <t>Rental Fee</t>
+  </si>
+  <si>
+    <t>Confirm Your Pay</t>
+  </si>
+  <si>
+    <t>Điểm trả xe</t>
+  </si>
+  <si>
+    <t>Phí thuê xe</t>
+  </si>
+  <si>
+    <t>Tổng cộng</t>
+  </si>
+  <si>
+    <t>Xác nhận thanh toán</t>
+  </si>
+  <si>
+    <t>ChangeBtn</t>
+  </si>
+  <si>
+    <t>Change</t>
+  </si>
+  <si>
+    <t>Thay đổi</t>
+  </si>
+  <si>
+    <t>SaveBtn</t>
+  </si>
+  <si>
+    <t>Save</t>
+  </si>
+  <si>
+    <t>Lưu</t>
+  </si>
+  <si>
+    <t>Pay Now</t>
+  </si>
+  <si>
+    <t>PayBtn</t>
+  </si>
+  <si>
+    <t>Trip Completed Successfully!</t>
+  </si>
+  <si>
+    <t>Thank you for riding with us. Please complete your payment.</t>
+  </si>
+  <si>
+    <t>Pickup Location</t>
+  </si>
+  <si>
+    <t>Return Location</t>
+  </si>
+  <si>
+    <t>Duration</t>
+  </si>
+  <si>
+    <t>Rate</t>
+  </si>
+  <si>
+    <t>Payment Breakdown</t>
+  </si>
+  <si>
+    <t>PAYMENT VIA</t>
+  </si>
+  <si>
+    <t>Transfer Information</t>
+  </si>
+  <si>
+    <t>Content:</t>
+  </si>
+  <si>
+    <t>Payment:</t>
+  </si>
+  <si>
+    <t>Please keep this page open to confirm your payment.</t>
+  </si>
+  <si>
+    <t>I Have Paid</t>
+  </si>
+  <si>
+    <t>TripSuccessTitle</t>
+  </si>
+  <si>
+    <t>TripSuccessDesc</t>
+  </si>
+  <si>
+    <t>VehicleLabel</t>
+  </si>
+  <si>
+    <t>PaymentMethodLabel</t>
+  </si>
+  <si>
+    <t>ContentLabel</t>
+  </si>
+  <si>
+    <t>AmountLabel</t>
+  </si>
+  <si>
+    <t>Chuyến đi hoàn tất!</t>
+  </si>
+  <si>
+    <t>Cảm ơn bạn đã đồng hành. Vui lòng thanh toán.</t>
+  </si>
+  <si>
+    <t>Phương tiện số</t>
+  </si>
+  <si>
+    <t>Điểm nhận xe</t>
+  </si>
+  <si>
+    <t>Đơn giá</t>
+  </si>
+  <si>
+    <t>Chi tiết thanh toán</t>
+  </si>
+  <si>
+    <t>THANH TOÁN QUA</t>
+  </si>
+  <si>
+    <t>Thông tin chuyển khoản</t>
+  </si>
+  <si>
+    <t>Nội dung:</t>
+  </si>
+  <si>
+    <t>Số tiền:</t>
+  </si>
+  <si>
+    <t>Vui lòng giữ trang này để xác nhận.</t>
+  </si>
+  <si>
+    <t>Tôi đã thanh toán</t>
+  </si>
+  <si>
+    <t>PaymentPickUp</t>
+  </si>
+  <si>
+    <t>PaymentReturnStation</t>
+  </si>
+  <si>
+    <t>RideDuration</t>
+  </si>
+  <si>
+    <t>RateLabel</t>
+  </si>
+  <si>
+    <t>PaymentBreakdown</t>
+  </si>
+  <si>
+    <t>RentalFeeLabel</t>
+  </si>
+  <si>
+    <t>PaymentHeader</t>
+  </si>
+  <si>
+    <t>PaymentSecureTitle</t>
+  </si>
+  <si>
+    <t>PaymentSecureDesc</t>
+  </si>
+  <si>
+    <t>ConfirmPaidBtn</t>
+  </si>
+  <si>
+    <t>Thanh Toán Ngay</t>
+  </si>
+  <si>
+    <t>SecUnit</t>
+  </si>
+  <si>
+    <t>sec</t>
+  </si>
+  <si>
+    <t>giây</t>
+  </si>
+  <si>
+    <t>SuccessHeader</t>
+  </si>
+  <si>
+    <t>SuccessSubHeader</t>
+  </si>
+  <si>
+    <t>TotalPaidLabel</t>
+  </si>
+  <si>
+    <t>ThankYouMsg</t>
+  </si>
+  <si>
+    <t>MethodLabel</t>
+  </si>
+  <si>
+    <t>TransactionIDLabel</t>
+  </si>
+  <si>
+    <t>DateLabel</t>
+  </si>
+  <si>
+    <t>BackHomeBtn</t>
+  </si>
+  <si>
+    <t>ViewHistoryBtn</t>
+  </si>
+  <si>
+    <t>Thanh toán thành công!</t>
+  </si>
+  <si>
+    <t>Giao dịch của bạn đã được xử lý hoàn tất.</t>
+  </si>
+  <si>
+    <t>Cảm ơn bạn đã đồng hành cùng</t>
+  </si>
+  <si>
+    <t>Mã giao dịch</t>
+  </si>
+  <si>
+    <t>Ngày thực hiện</t>
+  </si>
+  <si>
+    <t>Về trang chủ</t>
+  </si>
+  <si>
+    <t>Xem lịch sử</t>
+  </si>
+  <si>
+    <t>Payment Successful!</t>
+  </si>
+  <si>
+    <t>Your transaction has been processed successfully.</t>
+  </si>
+  <si>
+    <t>Total Amount Paid</t>
+  </si>
+  <si>
+    <t>Thank you for riding with</t>
+  </si>
+  <si>
+    <t>Method</t>
+  </si>
+  <si>
+    <t>Transaction ID</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Back Home</t>
+  </si>
+  <si>
+    <t>View History</t>
+  </si>
+  <si>
+    <t>Tổng tiền thanh toán</t>
+  </si>
+  <si>
+    <t>Thuê xe</t>
   </si>
 </sst>
 </file>
@@ -1934,7 +2189,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G176"/>
+  <dimension ref="A1:G205"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
@@ -2043,7 +2298,7 @@
         <v>10</v>
       </c>
       <c r="E5" t="s">
-        <v>16</v>
+        <v>492</v>
       </c>
       <c r="F5" t="s">
         <v>10</v>
@@ -4583,7 +4838,7 @@
         <v>438</v>
       </c>
       <c r="G153" t="s">
-        <v>457</v>
+        <v>604</v>
       </c>
     </row>
     <row r="154" spans="1:7" x14ac:dyDescent="0.3">
@@ -4600,7 +4855,7 @@
         <v>439</v>
       </c>
       <c r="G154" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="155" spans="1:7" x14ac:dyDescent="0.3">
@@ -4617,7 +4872,7 @@
         <v>440</v>
       </c>
       <c r="G155" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
     </row>
     <row r="156" spans="1:7" x14ac:dyDescent="0.3">
@@ -4628,13 +4883,13 @@
         <v>8</v>
       </c>
       <c r="C156" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="E156" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
       <c r="G156" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
     </row>
     <row r="157" spans="1:7" x14ac:dyDescent="0.3">
@@ -4645,13 +4900,13 @@
         <v>8</v>
       </c>
       <c r="C157" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
       <c r="E157" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="G157" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
     </row>
     <row r="158" spans="1:7" x14ac:dyDescent="0.3">
@@ -4662,13 +4917,13 @@
         <v>8</v>
       </c>
       <c r="C158" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="E158" t="s">
         <v>434</v>
       </c>
       <c r="G158" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
     </row>
     <row r="159" spans="1:7" x14ac:dyDescent="0.3">
@@ -4679,13 +4934,13 @@
         <v>8</v>
       </c>
       <c r="C159" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="E159" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
       <c r="G159" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
     </row>
     <row r="160" spans="1:7" x14ac:dyDescent="0.3">
@@ -4696,13 +4951,13 @@
         <v>8</v>
       </c>
       <c r="C160" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="E160" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="G160" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
     </row>
     <row r="161" spans="1:7" x14ac:dyDescent="0.3">
@@ -4713,13 +4968,13 @@
         <v>8</v>
       </c>
       <c r="C161" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="E161" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
       <c r="G161" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
     </row>
     <row r="162" spans="1:7" x14ac:dyDescent="0.3">
@@ -4730,10 +4985,10 @@
         <v>8</v>
       </c>
       <c r="C162" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="E162" t="s">
-        <v>497</v>
+        <v>495</v>
       </c>
       <c r="G162" t="s">
         <v>333</v>
@@ -4747,13 +5002,13 @@
         <v>8</v>
       </c>
       <c r="C163" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="E163" t="s">
-        <v>498</v>
+        <v>496</v>
       </c>
       <c r="G163" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
     </row>
     <row r="164" spans="1:7" x14ac:dyDescent="0.3">
@@ -4764,13 +5019,13 @@
         <v>8</v>
       </c>
       <c r="C164" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="E164" t="s">
-        <v>499</v>
+        <v>497</v>
       </c>
       <c r="G164" t="s">
-        <v>484</v>
+        <v>523</v>
       </c>
     </row>
     <row r="165" spans="1:7" x14ac:dyDescent="0.3">
@@ -4781,13 +5036,13 @@
         <v>8</v>
       </c>
       <c r="C165" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="E165" t="s">
-        <v>500</v>
+        <v>498</v>
       </c>
       <c r="G165" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
     </row>
     <row r="166" spans="1:7" x14ac:dyDescent="0.3">
@@ -4798,13 +5053,13 @@
         <v>8</v>
       </c>
       <c r="C166" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="E166" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
       <c r="G166" t="s">
-        <v>509</v>
+        <v>507</v>
       </c>
     </row>
     <row r="167" spans="1:7" x14ac:dyDescent="0.3">
@@ -4815,13 +5070,13 @@
         <v>8</v>
       </c>
       <c r="C167" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="E167" t="s">
-        <v>501</v>
+        <v>499</v>
       </c>
       <c r="G167" t="s">
-        <v>486</v>
+        <v>484</v>
       </c>
     </row>
     <row r="168" spans="1:7" x14ac:dyDescent="0.3">
@@ -4832,13 +5087,13 @@
         <v>8</v>
       </c>
       <c r="C168" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="E168" t="s">
-        <v>502</v>
+        <v>500</v>
       </c>
       <c r="G168" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
     </row>
     <row r="169" spans="1:7" x14ac:dyDescent="0.3">
@@ -4849,13 +5104,13 @@
         <v>8</v>
       </c>
       <c r="C169" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="E169" t="s">
-        <v>503</v>
+        <v>501</v>
       </c>
       <c r="G169" t="s">
-        <v>488</v>
+        <v>486</v>
       </c>
     </row>
     <row r="170" spans="1:7" x14ac:dyDescent="0.3">
@@ -4866,13 +5121,13 @@
         <v>8</v>
       </c>
       <c r="C170" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="E170" t="s">
-        <v>504</v>
+        <v>502</v>
       </c>
       <c r="G170" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
     </row>
     <row r="171" spans="1:7" x14ac:dyDescent="0.3">
@@ -4883,13 +5138,13 @@
         <v>8</v>
       </c>
       <c r="C171" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="E171" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
       <c r="G171" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
     </row>
     <row r="172" spans="1:7" x14ac:dyDescent="0.3">
@@ -4900,13 +5155,13 @@
         <v>8</v>
       </c>
       <c r="C172" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="E172" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
       <c r="G172" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
     </row>
     <row r="173" spans="1:7" x14ac:dyDescent="0.3">
@@ -4917,13 +5172,13 @@
         <v>8</v>
       </c>
       <c r="C173" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="E173" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="G173" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
     </row>
     <row r="174" spans="1:7" x14ac:dyDescent="0.3">
@@ -4934,13 +5189,13 @@
         <v>8</v>
       </c>
       <c r="C174" t="s">
+        <v>509</v>
+      </c>
+      <c r="E174" t="s">
         <v>511</v>
       </c>
-      <c r="E174" t="s">
-        <v>513</v>
-      </c>
       <c r="G174" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
     </row>
     <row r="175" spans="1:7" x14ac:dyDescent="0.3">
@@ -4951,13 +5206,13 @@
         <v>8</v>
       </c>
       <c r="C175" t="s">
+        <v>512</v>
+      </c>
+      <c r="E175" t="s">
         <v>514</v>
       </c>
-      <c r="E175" t="s">
-        <v>516</v>
-      </c>
       <c r="G175" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
     </row>
     <row r="176" spans="1:7" x14ac:dyDescent="0.3">
@@ -4968,13 +5223,506 @@
         <v>8</v>
       </c>
       <c r="C176" t="s">
+        <v>515</v>
+      </c>
+      <c r="E176" t="s">
         <v>517</v>
       </c>
-      <c r="E176" t="s">
+      <c r="G176" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="177" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A177" t="s">
+        <v>7</v>
+      </c>
+      <c r="B177" t="s">
+        <v>8</v>
+      </c>
+      <c r="C177" t="s">
+        <v>546</v>
+      </c>
+      <c r="E177" t="s">
+        <v>533</v>
+      </c>
+      <c r="G177" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="178" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A178" t="s">
+        <v>7</v>
+      </c>
+      <c r="B178" t="s">
+        <v>8</v>
+      </c>
+      <c r="C178" t="s">
+        <v>547</v>
+      </c>
+      <c r="E178" t="s">
+        <v>534</v>
+      </c>
+      <c r="G178" t="s">
+        <v>553</v>
+      </c>
+    </row>
+    <row r="179" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A179" t="s">
+        <v>7</v>
+      </c>
+      <c r="B179" t="s">
+        <v>8</v>
+      </c>
+      <c r="C179" t="s">
+        <v>548</v>
+      </c>
+      <c r="E179" t="s">
+        <v>518</v>
+      </c>
+      <c r="G179" t="s">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="180" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A180" t="s">
+        <v>7</v>
+      </c>
+      <c r="B180" t="s">
+        <v>8</v>
+      </c>
+      <c r="C180" t="s">
+        <v>564</v>
+      </c>
+      <c r="E180" t="s">
+        <v>535</v>
+      </c>
+      <c r="G180" t="s">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="181" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A181" t="s">
+        <v>7</v>
+      </c>
+      <c r="B181" t="s">
+        <v>8</v>
+      </c>
+      <c r="C181" t="s">
+        <v>565</v>
+      </c>
+      <c r="E181" t="s">
+        <v>536</v>
+      </c>
+      <c r="G181" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="182" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A182" t="s">
+        <v>7</v>
+      </c>
+      <c r="B182" t="s">
+        <v>8</v>
+      </c>
+      <c r="C182" t="s">
+        <v>566</v>
+      </c>
+      <c r="E182" t="s">
+        <v>537</v>
+      </c>
+      <c r="G182" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="183" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A183" t="s">
+        <v>7</v>
+      </c>
+      <c r="B183" t="s">
+        <v>8</v>
+      </c>
+      <c r="C183" t="s">
+        <v>567</v>
+      </c>
+      <c r="E183" t="s">
+        <v>538</v>
+      </c>
+      <c r="G183" t="s">
+        <v>556</v>
+      </c>
+    </row>
+    <row r="184" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A184" t="s">
+        <v>7</v>
+      </c>
+      <c r="B184" t="s">
+        <v>8</v>
+      </c>
+      <c r="C184" t="s">
+        <v>568</v>
+      </c>
+      <c r="E184" t="s">
+        <v>539</v>
+      </c>
+      <c r="G184" t="s">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="185" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A185" t="s">
+        <v>7</v>
+      </c>
+      <c r="B185" t="s">
+        <v>8</v>
+      </c>
+      <c r="C185" t="s">
+        <v>569</v>
+      </c>
+      <c r="E185" t="s">
         <v>519</v>
       </c>
-      <c r="G176" t="s">
-        <v>518</v>
+      <c r="G185" t="s">
+        <v>522</v>
+      </c>
+    </row>
+    <row r="186" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A186" t="s">
+        <v>7</v>
+      </c>
+      <c r="B186" t="s">
+        <v>8</v>
+      </c>
+      <c r="C186" t="s">
+        <v>549</v>
+      </c>
+      <c r="E186" t="s">
+        <v>540</v>
+      </c>
+      <c r="G186" t="s">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="187" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A187" t="s">
+        <v>7</v>
+      </c>
+      <c r="B187" t="s">
+        <v>8</v>
+      </c>
+      <c r="C187" t="s">
+        <v>570</v>
+      </c>
+      <c r="E187" t="s">
+        <v>520</v>
+      </c>
+      <c r="G187" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="188" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A188" t="s">
+        <v>7</v>
+      </c>
+      <c r="B188" t="s">
+        <v>8</v>
+      </c>
+      <c r="C188" t="s">
+        <v>571</v>
+      </c>
+      <c r="E188" t="s">
+        <v>541</v>
+      </c>
+      <c r="G188" t="s">
+        <v>559</v>
+      </c>
+    </row>
+    <row r="189" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A189" t="s">
+        <v>7</v>
+      </c>
+      <c r="B189" t="s">
+        <v>8</v>
+      </c>
+      <c r="C189" t="s">
+        <v>550</v>
+      </c>
+      <c r="E189" t="s">
+        <v>542</v>
+      </c>
+      <c r="G189" t="s">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="190" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A190" t="s">
+        <v>7</v>
+      </c>
+      <c r="B190" t="s">
+        <v>8</v>
+      </c>
+      <c r="C190" t="s">
+        <v>551</v>
+      </c>
+      <c r="E190" t="s">
+        <v>543</v>
+      </c>
+      <c r="G190" t="s">
+        <v>561</v>
+      </c>
+    </row>
+    <row r="191" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A191" t="s">
+        <v>7</v>
+      </c>
+      <c r="B191" t="s">
+        <v>8</v>
+      </c>
+      <c r="C191" t="s">
+        <v>572</v>
+      </c>
+      <c r="E191" t="s">
+        <v>544</v>
+      </c>
+      <c r="G191" t="s">
+        <v>562</v>
+      </c>
+    </row>
+    <row r="192" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A192" t="s">
+        <v>7</v>
+      </c>
+      <c r="B192" t="s">
+        <v>8</v>
+      </c>
+      <c r="C192" t="s">
+        <v>573</v>
+      </c>
+      <c r="E192" t="s">
+        <v>545</v>
+      </c>
+      <c r="G192" t="s">
+        <v>563</v>
+      </c>
+    </row>
+    <row r="193" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A193" t="s">
+        <v>7</v>
+      </c>
+      <c r="B193" t="s">
+        <v>8</v>
+      </c>
+      <c r="C193" t="s">
+        <v>525</v>
+      </c>
+      <c r="E193" t="s">
+        <v>526</v>
+      </c>
+      <c r="G193" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="194" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A194" t="s">
+        <v>7</v>
+      </c>
+      <c r="B194" t="s">
+        <v>8</v>
+      </c>
+      <c r="C194" t="s">
+        <v>528</v>
+      </c>
+      <c r="E194" t="s">
+        <v>529</v>
+      </c>
+      <c r="G194" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="195" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A195" t="s">
+        <v>7</v>
+      </c>
+      <c r="B195" t="s">
+        <v>8</v>
+      </c>
+      <c r="C195" t="s">
+        <v>532</v>
+      </c>
+      <c r="E195" t="s">
+        <v>531</v>
+      </c>
+      <c r="G195" t="s">
+        <v>574</v>
+      </c>
+    </row>
+    <row r="196" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A196" t="s">
+        <v>7</v>
+      </c>
+      <c r="B196" t="s">
+        <v>8</v>
+      </c>
+      <c r="C196" t="s">
+        <v>575</v>
+      </c>
+      <c r="E196" t="s">
+        <v>576</v>
+      </c>
+      <c r="G196" t="s">
+        <v>577</v>
+      </c>
+    </row>
+    <row r="197" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A197" t="s">
+        <v>7</v>
+      </c>
+      <c r="B197" t="s">
+        <v>8</v>
+      </c>
+      <c r="C197" t="s">
+        <v>578</v>
+      </c>
+      <c r="E197" t="s">
+        <v>594</v>
+      </c>
+      <c r="G197" t="s">
+        <v>587</v>
+      </c>
+    </row>
+    <row r="198" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A198" t="s">
+        <v>7</v>
+      </c>
+      <c r="B198" t="s">
+        <v>8</v>
+      </c>
+      <c r="C198" t="s">
+        <v>579</v>
+      </c>
+      <c r="E198" t="s">
+        <v>595</v>
+      </c>
+      <c r="G198" t="s">
+        <v>588</v>
+      </c>
+    </row>
+    <row r="199" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A199" t="s">
+        <v>7</v>
+      </c>
+      <c r="B199" t="s">
+        <v>8</v>
+      </c>
+      <c r="C199" t="s">
+        <v>580</v>
+      </c>
+      <c r="E199" t="s">
+        <v>596</v>
+      </c>
+      <c r="G199" t="s">
+        <v>603</v>
+      </c>
+    </row>
+    <row r="200" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A200" t="s">
+        <v>7</v>
+      </c>
+      <c r="B200" t="s">
+        <v>8</v>
+      </c>
+      <c r="C200" t="s">
+        <v>581</v>
+      </c>
+      <c r="E200" t="s">
+        <v>597</v>
+      </c>
+      <c r="G200" t="s">
+        <v>589</v>
+      </c>
+    </row>
+    <row r="201" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A201" t="s">
+        <v>7</v>
+      </c>
+      <c r="B201" t="s">
+        <v>8</v>
+      </c>
+      <c r="C201" t="s">
+        <v>582</v>
+      </c>
+      <c r="E201" t="s">
+        <v>598</v>
+      </c>
+      <c r="G201" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="202" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A202" t="s">
+        <v>7</v>
+      </c>
+      <c r="B202" t="s">
+        <v>8</v>
+      </c>
+      <c r="C202" t="s">
+        <v>583</v>
+      </c>
+      <c r="E202" t="s">
+        <v>599</v>
+      </c>
+      <c r="G202" t="s">
+        <v>590</v>
+      </c>
+    </row>
+    <row r="203" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A203" t="s">
+        <v>7</v>
+      </c>
+      <c r="B203" t="s">
+        <v>8</v>
+      </c>
+      <c r="C203" t="s">
+        <v>584</v>
+      </c>
+      <c r="E203" t="s">
+        <v>600</v>
+      </c>
+      <c r="G203" t="s">
+        <v>591</v>
+      </c>
+    </row>
+    <row r="204" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A204" t="s">
+        <v>7</v>
+      </c>
+      <c r="B204" t="s">
+        <v>8</v>
+      </c>
+      <c r="C204" t="s">
+        <v>585</v>
+      </c>
+      <c r="E204" t="s">
+        <v>601</v>
+      </c>
+      <c r="G204" t="s">
+        <v>592</v>
+      </c>
+    </row>
+    <row r="205" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A205" t="s">
+        <v>7</v>
+      </c>
+      <c r="B205" t="s">
+        <v>8</v>
+      </c>
+      <c r="C205" t="s">
+        <v>586</v>
+      </c>
+      <c r="E205" t="s">
+        <v>602</v>
+      </c>
+      <c r="G205" t="s">
+        <v>593</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Done: language for rental, user
</commit_message>
<xml_diff>
--- a/language.xlsx
+++ b/language.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\OneDrive\Documents\SaigonRide_Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F639CE3-17BA-4DA7-86C0-8BD7C3C4544F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0F97013-F3D0-461C-BACE-5EF659136476}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1041" uniqueCount="605">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1276" uniqueCount="732">
   <si>
     <t>Project</t>
   </si>
@@ -1651,9 +1651,6 @@
     <t>Content:</t>
   </si>
   <si>
-    <t>Payment:</t>
-  </si>
-  <si>
     <t>Please keep this page open to confirm your payment.</t>
   </si>
   <si>
@@ -1705,9 +1702,6 @@
     <t>Nội dung:</t>
   </si>
   <si>
-    <t>Số tiền:</t>
-  </si>
-  <si>
     <t>Vui lòng giữ trang này để xác nhận.</t>
   </si>
   <si>
@@ -1835,6 +1829,393 @@
   </si>
   <si>
     <t>Thuê xe</t>
+  </si>
+  <si>
+    <t>TripHistoryTitle</t>
+  </si>
+  <si>
+    <t>TotalTrips</t>
+  </si>
+  <si>
+    <t>ColVehicle</t>
+  </si>
+  <si>
+    <t>ColPlateNumber</t>
+  </si>
+  <si>
+    <t>ColBilling</t>
+  </si>
+  <si>
+    <t>MinsUnit</t>
+  </si>
+  <si>
+    <t>SavedAmount</t>
+  </si>
+  <si>
+    <t>SuccessStatus</t>
+  </si>
+  <si>
+    <t>Trip History</t>
+  </si>
+  <si>
+    <t>Total: {0} Trips</t>
+  </si>
+  <si>
+    <t>Plate Number</t>
+  </si>
+  <si>
+    <t>Billing</t>
+  </si>
+  <si>
+    <t>mins</t>
+  </si>
+  <si>
+    <t>Saved {0}</t>
+  </si>
+  <si>
+    <t>SUCCESS</t>
+  </si>
+  <si>
+    <t>Lịch sử chuyến đi</t>
+  </si>
+  <si>
+    <t>Tổng cộng: {0} chuyến</t>
+  </si>
+  <si>
+    <t>Phương tiện</t>
+  </si>
+  <si>
+    <t>Thanh toán</t>
+  </si>
+  <si>
+    <t>Đã giảm {0}</t>
+  </si>
+  <si>
+    <t>THÀNH CÔNG</t>
+  </si>
+  <si>
+    <t>ColDuration</t>
+  </si>
+  <si>
+    <t>ColStatus</t>
+  </si>
+  <si>
+    <t>ColDate</t>
+  </si>
+  <si>
+    <t>TransactionSubTitle</t>
+  </si>
+  <si>
+    <t>TotalActivities</t>
+  </si>
+  <si>
+    <t>ColActivity</t>
+  </si>
+  <si>
+    <t>WalletTopUp</t>
+  </si>
+  <si>
+    <t>RidePayment</t>
+  </si>
+  <si>
+    <t>MyTransactions</t>
+  </si>
+  <si>
+    <t>My Transactions</t>
+  </si>
+  <si>
+    <t>Track your wallet history and payments</t>
+  </si>
+  <si>
+    <t>Total Activities</t>
+  </si>
+  <si>
+    <t>Activity</t>
+  </si>
+  <si>
+    <t>Wallet Top Up</t>
+  </si>
+  <si>
+    <t>Ride Payment</t>
+  </si>
+  <si>
+    <t>Giao dịch của tôi</t>
+  </si>
+  <si>
+    <t>Theo dõi lịch sử ví và thanh toán</t>
+  </si>
+  <si>
+    <t>Tổng hoạt động</t>
+  </si>
+  <si>
+    <t>Hoạt động</t>
+  </si>
+  <si>
+    <t>Nạp tiền vào ví</t>
+  </si>
+  <si>
+    <t>Thanh toán chuyến đi</t>
+  </si>
+  <si>
+    <t>Payment</t>
+  </si>
+  <si>
+    <t>ProfileTitle</t>
+  </si>
+  <si>
+    <t>ProfileSubTitle</t>
+  </si>
+  <si>
+    <t>StatusActive</t>
+  </si>
+  <si>
+    <t>StatusLocked</t>
+  </si>
+  <si>
+    <t>AccountTypeLabel</t>
+  </si>
+  <si>
+    <t>RoleLabel</t>
+  </si>
+  <si>
+    <t>AvailableBalance</t>
+  </si>
+  <si>
+    <t>TopUpPrompt</t>
+  </si>
+  <si>
+    <t>TopUpDesc</t>
+  </si>
+  <si>
+    <t>TopUpBtn</t>
+  </si>
+  <si>
+    <t>My Profile</t>
+  </si>
+  <si>
+    <t>Manage your personal account information</t>
+  </si>
+  <si>
+    <t>Active</t>
+  </si>
+  <si>
+    <t>Locked</t>
+  </si>
+  <si>
+    <t>Account Type</t>
+  </si>
+  <si>
+    <t>Role</t>
+  </si>
+  <si>
+    <t>Available Balance</t>
+  </si>
+  <si>
+    <t>Need more balance?</t>
+  </si>
+  <si>
+    <t>Add funds to your wallet to continue using our services</t>
+  </si>
+  <si>
+    <t>Top Up Now</t>
+  </si>
+  <si>
+    <t>Hồ sơ của tôi</t>
+  </si>
+  <si>
+    <t>Quản lý thông tin tài khoản cá nhân</t>
+  </si>
+  <si>
+    <t>Đã bị khóa</t>
+  </si>
+  <si>
+    <t>Loại tài khoản</t>
+  </si>
+  <si>
+    <t>Vai trò</t>
+  </si>
+  <si>
+    <t>Số dư khả dụng</t>
+  </si>
+  <si>
+    <t>Bạn cần thêm số dư?</t>
+  </si>
+  <si>
+    <t>Nạp thêm tiền vào ví để tiếp tục sử dụng dịch vụ</t>
+  </si>
+  <si>
+    <t>Nạp tiền ngay</t>
+  </si>
+  <si>
+    <t>Local</t>
+  </si>
+  <si>
+    <t>RoleUser</t>
+  </si>
+  <si>
+    <t>User</t>
+  </si>
+  <si>
+    <t>Người dùng</t>
+  </si>
+  <si>
+    <t>TopUpTitle</t>
+  </si>
+  <si>
+    <t>TopUpSubTitle</t>
+  </si>
+  <si>
+    <t>RechargeAmountLabel</t>
+  </si>
+  <si>
+    <t>MinDepositMsg</t>
+  </si>
+  <si>
+    <t>ConfirmTopUpBtn</t>
+  </si>
+  <si>
+    <t>SecuredSSL</t>
+  </si>
+  <si>
+    <t>Top Up Wallet</t>
+  </si>
+  <si>
+    <t>Quickly add funds to your account</t>
+  </si>
+  <si>
+    <t>Recharge Amount</t>
+  </si>
+  <si>
+    <t>Min deposit: {0} VND</t>
+  </si>
+  <si>
+    <t>Confirm Top Up</t>
+  </si>
+  <si>
+    <t>Secured 256-bit SSL connection</t>
+  </si>
+  <si>
+    <t>Nạp tiền nhanh chóng vào tài khoản</t>
+  </si>
+  <si>
+    <t>Số tiền nạp</t>
+  </si>
+  <si>
+    <t>Nạp tối thiểu: {0} VND</t>
+  </si>
+  <si>
+    <t>Xác nhận nạp tiền</t>
+  </si>
+  <si>
+    <t>Kết nối SSL 256-bit an toàn</t>
+  </si>
+  <si>
+    <t>PaymentMethodCash</t>
+  </si>
+  <si>
+    <t>Tiền mặt</t>
+  </si>
+  <si>
+    <t>Cash</t>
+  </si>
+  <si>
+    <t>EmailRequired</t>
+  </si>
+  <si>
+    <t>InvalidEmail</t>
+  </si>
+  <si>
+    <t>PasswordRequired</t>
+  </si>
+  <si>
+    <t>ConfirmPasswordRequired</t>
+  </si>
+  <si>
+    <t>PasswordMismatch</t>
+  </si>
+  <si>
+    <t>PassMinLength</t>
+  </si>
+  <si>
+    <t>PassUppercase</t>
+  </si>
+  <si>
+    <t>PassNumber</t>
+  </si>
+  <si>
+    <t>Mật khẩu phải có ít nhất 8 ký tự.</t>
+  </si>
+  <si>
+    <t>Mật khẩu phải có ít nhất 1 chữ hoa.</t>
+  </si>
+  <si>
+    <t>Mật khẩu phải có ít nhất 1 chữ số.</t>
+  </si>
+  <si>
+    <t>Invalid email format.</t>
+  </si>
+  <si>
+    <t>Please confirm your password.</t>
+  </si>
+  <si>
+    <t>Passwords do not match.</t>
+  </si>
+  <si>
+    <t>Password must contain at least 1 uppercase letter.</t>
+  </si>
+  <si>
+    <t>Password must contain at least 1 number.</t>
+  </si>
+  <si>
+    <t>FullNameRequired</t>
+  </si>
+  <si>
+    <t>FullNameMinLength</t>
+  </si>
+  <si>
+    <t>EmailNoSpaces</t>
+  </si>
+  <si>
+    <t>Vui lòng nhập họ tên.</t>
+  </si>
+  <si>
+    <t>Họ tên phải từ 3 ký tự trở lên.</t>
+  </si>
+  <si>
+    <t>Vui lòng nhập email.</t>
+  </si>
+  <si>
+    <t>Định dạng email không hợp lệ.</t>
+  </si>
+  <si>
+    <t>Email không được chứa khoảng trắng.</t>
+  </si>
+  <si>
+    <t>Vui lòng nhập mật khẩu.</t>
+  </si>
+  <si>
+    <t>Vui lòng xác nhận mật khẩu.</t>
+  </si>
+  <si>
+    <t>Mật khẩu không trùng khớp.</t>
+  </si>
+  <si>
+    <t>Full name is required.</t>
+  </si>
+  <si>
+    <t>Full name must be at least 3 characters.</t>
+  </si>
+  <si>
+    <t>Email is required.</t>
+  </si>
+  <si>
+    <t>Email cannot contain spaces.</t>
+  </si>
+  <si>
+    <t>Password is required.</t>
+  </si>
+  <si>
+    <t>Password must be at least 8 characters.</t>
   </si>
 </sst>
 </file>
@@ -2189,7 +2570,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G205"/>
+  <dimension ref="A1:G252"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
@@ -4838,7 +5219,7 @@
         <v>438</v>
       </c>
       <c r="G153" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
     </row>
     <row r="154" spans="1:7" x14ac:dyDescent="0.3">
@@ -5240,13 +5621,13 @@
         <v>8</v>
       </c>
       <c r="C177" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="E177" t="s">
         <v>533</v>
       </c>
       <c r="G177" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
     </row>
     <row r="178" spans="1:7" x14ac:dyDescent="0.3">
@@ -5257,13 +5638,13 @@
         <v>8</v>
       </c>
       <c r="C178" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="E178" t="s">
         <v>534</v>
       </c>
       <c r="G178" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
     </row>
     <row r="179" spans="1:7" x14ac:dyDescent="0.3">
@@ -5274,13 +5655,13 @@
         <v>8</v>
       </c>
       <c r="C179" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="E179" t="s">
         <v>518</v>
       </c>
       <c r="G179" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
     </row>
     <row r="180" spans="1:7" x14ac:dyDescent="0.3">
@@ -5291,13 +5672,13 @@
         <v>8</v>
       </c>
       <c r="C180" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
       <c r="E180" t="s">
         <v>535</v>
       </c>
       <c r="G180" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
     </row>
     <row r="181" spans="1:7" x14ac:dyDescent="0.3">
@@ -5308,7 +5689,7 @@
         <v>8</v>
       </c>
       <c r="C181" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="E181" t="s">
         <v>536</v>
@@ -5325,7 +5706,7 @@
         <v>8</v>
       </c>
       <c r="C182" t="s">
-        <v>566</v>
+        <v>564</v>
       </c>
       <c r="E182" t="s">
         <v>537</v>
@@ -5342,13 +5723,13 @@
         <v>8</v>
       </c>
       <c r="C183" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
       <c r="E183" t="s">
         <v>538</v>
       </c>
       <c r="G183" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
     </row>
     <row r="184" spans="1:7" x14ac:dyDescent="0.3">
@@ -5359,13 +5740,13 @@
         <v>8</v>
       </c>
       <c r="C184" t="s">
-        <v>568</v>
+        <v>566</v>
       </c>
       <c r="E184" t="s">
         <v>539</v>
       </c>
       <c r="G184" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
     </row>
     <row r="185" spans="1:7" x14ac:dyDescent="0.3">
@@ -5376,7 +5757,7 @@
         <v>8</v>
       </c>
       <c r="C185" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
       <c r="E185" t="s">
         <v>519</v>
@@ -5393,13 +5774,13 @@
         <v>8</v>
       </c>
       <c r="C186" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="E186" t="s">
         <v>540</v>
       </c>
       <c r="G186" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
     </row>
     <row r="187" spans="1:7" x14ac:dyDescent="0.3">
@@ -5410,7 +5791,7 @@
         <v>8</v>
       </c>
       <c r="C187" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="E187" t="s">
         <v>520</v>
@@ -5427,13 +5808,13 @@
         <v>8</v>
       </c>
       <c r="C188" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="E188" t="s">
         <v>541</v>
       </c>
       <c r="G188" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
     </row>
     <row r="189" spans="1:7" x14ac:dyDescent="0.3">
@@ -5444,13 +5825,13 @@
         <v>8</v>
       </c>
       <c r="C189" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="E189" t="s">
         <v>542</v>
       </c>
       <c r="G189" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
     </row>
     <row r="190" spans="1:7" x14ac:dyDescent="0.3">
@@ -5461,13 +5842,13 @@
         <v>8</v>
       </c>
       <c r="C190" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="E190" t="s">
-        <v>543</v>
+        <v>645</v>
       </c>
       <c r="G190" t="s">
-        <v>561</v>
+        <v>308</v>
       </c>
     </row>
     <row r="191" spans="1:7" x14ac:dyDescent="0.3">
@@ -5478,13 +5859,13 @@
         <v>8</v>
       </c>
       <c r="C191" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="E191" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="G191" t="s">
-        <v>562</v>
+        <v>560</v>
       </c>
     </row>
     <row r="192" spans="1:7" x14ac:dyDescent="0.3">
@@ -5495,13 +5876,13 @@
         <v>8</v>
       </c>
       <c r="C192" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
       <c r="E192" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="G192" t="s">
-        <v>563</v>
+        <v>561</v>
       </c>
     </row>
     <row r="193" spans="1:7" x14ac:dyDescent="0.3">
@@ -5552,7 +5933,7 @@
         <v>531</v>
       </c>
       <c r="G195" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
     </row>
     <row r="196" spans="1:7" x14ac:dyDescent="0.3">
@@ -5563,13 +5944,13 @@
         <v>8</v>
       </c>
       <c r="C196" t="s">
+        <v>573</v>
+      </c>
+      <c r="E196" t="s">
+        <v>574</v>
+      </c>
+      <c r="G196" t="s">
         <v>575</v>
-      </c>
-      <c r="E196" t="s">
-        <v>576</v>
-      </c>
-      <c r="G196" t="s">
-        <v>577</v>
       </c>
     </row>
     <row r="197" spans="1:7" x14ac:dyDescent="0.3">
@@ -5580,13 +5961,13 @@
         <v>8</v>
       </c>
       <c r="C197" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="E197" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="G197" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
     </row>
     <row r="198" spans="1:7" x14ac:dyDescent="0.3">
@@ -5597,13 +5978,13 @@
         <v>8</v>
       </c>
       <c r="C198" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="E198" t="s">
-        <v>595</v>
+        <v>593</v>
       </c>
       <c r="G198" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
     </row>
     <row r="199" spans="1:7" x14ac:dyDescent="0.3">
@@ -5614,13 +5995,13 @@
         <v>8</v>
       </c>
       <c r="C199" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="E199" t="s">
-        <v>596</v>
+        <v>594</v>
       </c>
       <c r="G199" t="s">
-        <v>603</v>
+        <v>601</v>
       </c>
     </row>
     <row r="200" spans="1:7" x14ac:dyDescent="0.3">
@@ -5631,13 +6012,13 @@
         <v>8</v>
       </c>
       <c r="C200" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
       <c r="E200" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="G200" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
     </row>
     <row r="201" spans="1:7" x14ac:dyDescent="0.3">
@@ -5648,10 +6029,10 @@
         <v>8</v>
       </c>
       <c r="C201" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="E201" t="s">
-        <v>598</v>
+        <v>596</v>
       </c>
       <c r="G201" t="s">
         <v>516</v>
@@ -5665,13 +6046,13 @@
         <v>8</v>
       </c>
       <c r="C202" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="E202" t="s">
-        <v>599</v>
+        <v>597</v>
       </c>
       <c r="G202" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
     </row>
     <row r="203" spans="1:7" x14ac:dyDescent="0.3">
@@ -5682,13 +6063,13 @@
         <v>8</v>
       </c>
       <c r="C203" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="E203" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="G203" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
     </row>
     <row r="204" spans="1:7" x14ac:dyDescent="0.3">
@@ -5699,13 +6080,13 @@
         <v>8</v>
       </c>
       <c r="C204" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="E204" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="G204" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
     </row>
     <row r="205" spans="1:7" x14ac:dyDescent="0.3">
@@ -5716,13 +6097,812 @@
         <v>8</v>
       </c>
       <c r="C205" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="E205" t="s">
-        <v>602</v>
+        <v>600</v>
       </c>
       <c r="G205" t="s">
-        <v>593</v>
+        <v>591</v>
+      </c>
+    </row>
+    <row r="206" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A206" t="s">
+        <v>7</v>
+      </c>
+      <c r="B206" t="s">
+        <v>8</v>
+      </c>
+      <c r="C206" t="s">
+        <v>603</v>
+      </c>
+      <c r="E206" t="s">
+        <v>611</v>
+      </c>
+      <c r="G206" t="s">
+        <v>618</v>
+      </c>
+    </row>
+    <row r="207" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A207" t="s">
+        <v>7</v>
+      </c>
+      <c r="B207" t="s">
+        <v>8</v>
+      </c>
+      <c r="C207" t="s">
+        <v>604</v>
+      </c>
+      <c r="E207" t="s">
+        <v>612</v>
+      </c>
+      <c r="G207" t="s">
+        <v>619</v>
+      </c>
+    </row>
+    <row r="208" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A208" t="s">
+        <v>7</v>
+      </c>
+      <c r="B208" t="s">
+        <v>8</v>
+      </c>
+      <c r="C208" t="s">
+        <v>605</v>
+      </c>
+      <c r="E208" t="s">
+        <v>518</v>
+      </c>
+      <c r="G208" t="s">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="209" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A209" t="s">
+        <v>7</v>
+      </c>
+      <c r="B209" t="s">
+        <v>8</v>
+      </c>
+      <c r="C209" t="s">
+        <v>606</v>
+      </c>
+      <c r="E209" t="s">
+        <v>613</v>
+      </c>
+      <c r="G209" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="210" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A210" t="s">
+        <v>7</v>
+      </c>
+      <c r="B210" t="s">
+        <v>8</v>
+      </c>
+      <c r="C210" t="s">
+        <v>624</v>
+      </c>
+      <c r="E210" t="s">
+        <v>537</v>
+      </c>
+      <c r="G210" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="211" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A211" t="s">
+        <v>7</v>
+      </c>
+      <c r="B211" t="s">
+        <v>8</v>
+      </c>
+      <c r="C211" t="s">
+        <v>607</v>
+      </c>
+      <c r="E211" t="s">
+        <v>614</v>
+      </c>
+      <c r="G211" t="s">
+        <v>621</v>
+      </c>
+    </row>
+    <row r="212" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A212" t="s">
+        <v>7</v>
+      </c>
+      <c r="B212" t="s">
+        <v>8</v>
+      </c>
+      <c r="C212" t="s">
+        <v>625</v>
+      </c>
+      <c r="E212" t="s">
+        <v>437</v>
+      </c>
+      <c r="G212" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="213" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A213" t="s">
+        <v>7</v>
+      </c>
+      <c r="B213" t="s">
+        <v>8</v>
+      </c>
+      <c r="C213" t="s">
+        <v>626</v>
+      </c>
+      <c r="E213" t="s">
+        <v>598</v>
+      </c>
+      <c r="G213" t="s">
+        <v>589</v>
+      </c>
+    </row>
+    <row r="214" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A214" t="s">
+        <v>7</v>
+      </c>
+      <c r="B214" t="s">
+        <v>8</v>
+      </c>
+      <c r="C214" t="s">
+        <v>608</v>
+      </c>
+      <c r="E214" t="s">
+        <v>615</v>
+      </c>
+      <c r="G214" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="215" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A215" t="s">
+        <v>7</v>
+      </c>
+      <c r="B215" t="s">
+        <v>8</v>
+      </c>
+      <c r="C215" t="s">
+        <v>609</v>
+      </c>
+      <c r="E215" t="s">
+        <v>616</v>
+      </c>
+      <c r="G215" t="s">
+        <v>622</v>
+      </c>
+    </row>
+    <row r="216" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A216" t="s">
+        <v>7</v>
+      </c>
+      <c r="B216" t="s">
+        <v>8</v>
+      </c>
+      <c r="C216" t="s">
+        <v>610</v>
+      </c>
+      <c r="E216" t="s">
+        <v>617</v>
+      </c>
+      <c r="G216" t="s">
+        <v>623</v>
+      </c>
+    </row>
+    <row r="217" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A217" t="s">
+        <v>7</v>
+      </c>
+      <c r="B217" t="s">
+        <v>8</v>
+      </c>
+      <c r="C217" t="s">
+        <v>632</v>
+      </c>
+      <c r="E217" t="s">
+        <v>633</v>
+      </c>
+      <c r="G217" t="s">
+        <v>639</v>
+      </c>
+    </row>
+    <row r="218" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A218" t="s">
+        <v>7</v>
+      </c>
+      <c r="B218" t="s">
+        <v>8</v>
+      </c>
+      <c r="C218" t="s">
+        <v>627</v>
+      </c>
+      <c r="E218" t="s">
+        <v>634</v>
+      </c>
+      <c r="G218" t="s">
+        <v>640</v>
+      </c>
+    </row>
+    <row r="219" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A219" t="s">
+        <v>7</v>
+      </c>
+      <c r="B219" t="s">
+        <v>8</v>
+      </c>
+      <c r="C219" t="s">
+        <v>628</v>
+      </c>
+      <c r="E219" t="s">
+        <v>635</v>
+      </c>
+      <c r="G219" t="s">
+        <v>641</v>
+      </c>
+    </row>
+    <row r="220" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A220" t="s">
+        <v>7</v>
+      </c>
+      <c r="B220" t="s">
+        <v>8</v>
+      </c>
+      <c r="C220" t="s">
+        <v>629</v>
+      </c>
+      <c r="E220" t="s">
+        <v>636</v>
+      </c>
+      <c r="G220" t="s">
+        <v>642</v>
+      </c>
+    </row>
+    <row r="221" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A221" t="s">
+        <v>7</v>
+      </c>
+      <c r="B221" t="s">
+        <v>8</v>
+      </c>
+      <c r="C221" t="s">
+        <v>630</v>
+      </c>
+      <c r="E221" t="s">
+        <v>637</v>
+      </c>
+      <c r="G221" t="s">
+        <v>643</v>
+      </c>
+    </row>
+    <row r="222" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A222" t="s">
+        <v>7</v>
+      </c>
+      <c r="B222" t="s">
+        <v>8</v>
+      </c>
+      <c r="C222" t="s">
+        <v>631</v>
+      </c>
+      <c r="E222" t="s">
+        <v>638</v>
+      </c>
+      <c r="G222" t="s">
+        <v>644</v>
+      </c>
+    </row>
+    <row r="223" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A223" t="s">
+        <v>7</v>
+      </c>
+      <c r="B223" t="s">
+        <v>8</v>
+      </c>
+      <c r="C223" t="s">
+        <v>646</v>
+      </c>
+      <c r="E223" t="s">
+        <v>656</v>
+      </c>
+      <c r="G223" t="s">
+        <v>666</v>
+      </c>
+    </row>
+    <row r="224" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A224" t="s">
+        <v>7</v>
+      </c>
+      <c r="B224" t="s">
+        <v>8</v>
+      </c>
+      <c r="C224" t="s">
+        <v>647</v>
+      </c>
+      <c r="E224" t="s">
+        <v>657</v>
+      </c>
+      <c r="G224" t="s">
+        <v>667</v>
+      </c>
+    </row>
+    <row r="225" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A225" t="s">
+        <v>7</v>
+      </c>
+      <c r="B225" t="s">
+        <v>8</v>
+      </c>
+      <c r="C225" t="s">
+        <v>648</v>
+      </c>
+      <c r="E225" t="s">
+        <v>658</v>
+      </c>
+      <c r="G225" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="226" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A226" t="s">
+        <v>7</v>
+      </c>
+      <c r="B226" t="s">
+        <v>8</v>
+      </c>
+      <c r="C226" t="s">
+        <v>649</v>
+      </c>
+      <c r="E226" t="s">
+        <v>659</v>
+      </c>
+      <c r="G226" t="s">
+        <v>668</v>
+      </c>
+    </row>
+    <row r="227" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A227" t="s">
+        <v>7</v>
+      </c>
+      <c r="B227" t="s">
+        <v>8</v>
+      </c>
+      <c r="C227" t="s">
+        <v>650</v>
+      </c>
+      <c r="E227" t="s">
+        <v>660</v>
+      </c>
+      <c r="G227" t="s">
+        <v>669</v>
+      </c>
+    </row>
+    <row r="228" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A228" t="s">
+        <v>7</v>
+      </c>
+      <c r="B228" t="s">
+        <v>8</v>
+      </c>
+      <c r="C228" t="s">
+        <v>651</v>
+      </c>
+      <c r="E228" t="s">
+        <v>661</v>
+      </c>
+      <c r="G228" t="s">
+        <v>670</v>
+      </c>
+    </row>
+    <row r="229" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A229" t="s">
+        <v>7</v>
+      </c>
+      <c r="B229" t="s">
+        <v>8</v>
+      </c>
+      <c r="C229" t="s">
+        <v>652</v>
+      </c>
+      <c r="E229" t="s">
+        <v>662</v>
+      </c>
+      <c r="G229" t="s">
+        <v>671</v>
+      </c>
+    </row>
+    <row r="230" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A230" t="s">
+        <v>7</v>
+      </c>
+      <c r="B230" t="s">
+        <v>8</v>
+      </c>
+      <c r="C230" t="s">
+        <v>653</v>
+      </c>
+      <c r="E230" t="s">
+        <v>663</v>
+      </c>
+      <c r="G230" t="s">
+        <v>672</v>
+      </c>
+    </row>
+    <row r="231" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A231" t="s">
+        <v>7</v>
+      </c>
+      <c r="B231" t="s">
+        <v>8</v>
+      </c>
+      <c r="C231" t="s">
+        <v>654</v>
+      </c>
+      <c r="E231" t="s">
+        <v>664</v>
+      </c>
+      <c r="G231" t="s">
+        <v>673</v>
+      </c>
+    </row>
+    <row r="232" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A232" t="s">
+        <v>7</v>
+      </c>
+      <c r="B232" t="s">
+        <v>8</v>
+      </c>
+      <c r="C232" t="s">
+        <v>655</v>
+      </c>
+      <c r="E232" t="s">
+        <v>665</v>
+      </c>
+      <c r="G232" t="s">
+        <v>674</v>
+      </c>
+    </row>
+    <row r="233" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A233" t="s">
+        <v>7</v>
+      </c>
+      <c r="B233" t="s">
+        <v>8</v>
+      </c>
+      <c r="C233" t="s">
+        <v>675</v>
+      </c>
+      <c r="E233" t="s">
+        <v>675</v>
+      </c>
+      <c r="G233" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="234" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A234" t="s">
+        <v>7</v>
+      </c>
+      <c r="B234" t="s">
+        <v>8</v>
+      </c>
+      <c r="C234" t="s">
+        <v>676</v>
+      </c>
+      <c r="E234" t="s">
+        <v>677</v>
+      </c>
+      <c r="G234" t="s">
+        <v>678</v>
+      </c>
+    </row>
+    <row r="235" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A235" t="s">
+        <v>7</v>
+      </c>
+      <c r="B235" t="s">
+        <v>8</v>
+      </c>
+      <c r="C235" t="s">
+        <v>679</v>
+      </c>
+      <c r="E235" t="s">
+        <v>685</v>
+      </c>
+      <c r="G235" t="s">
+        <v>643</v>
+      </c>
+    </row>
+    <row r="236" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A236" t="s">
+        <v>7</v>
+      </c>
+      <c r="B236" t="s">
+        <v>8</v>
+      </c>
+      <c r="C236" t="s">
+        <v>680</v>
+      </c>
+      <c r="E236" t="s">
+        <v>686</v>
+      </c>
+      <c r="G236" t="s">
+        <v>691</v>
+      </c>
+    </row>
+    <row r="237" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A237" t="s">
+        <v>7</v>
+      </c>
+      <c r="B237" t="s">
+        <v>8</v>
+      </c>
+      <c r="C237" t="s">
+        <v>681</v>
+      </c>
+      <c r="E237" t="s">
+        <v>687</v>
+      </c>
+      <c r="G237" t="s">
+        <v>692</v>
+      </c>
+    </row>
+    <row r="238" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A238" t="s">
+        <v>7</v>
+      </c>
+      <c r="B238" t="s">
+        <v>8</v>
+      </c>
+      <c r="C238" t="s">
+        <v>682</v>
+      </c>
+      <c r="E238" t="s">
+        <v>688</v>
+      </c>
+      <c r="G238" t="s">
+        <v>693</v>
+      </c>
+    </row>
+    <row r="239" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A239" t="s">
+        <v>7</v>
+      </c>
+      <c r="B239" t="s">
+        <v>8</v>
+      </c>
+      <c r="C239" t="s">
+        <v>683</v>
+      </c>
+      <c r="E239" t="s">
+        <v>689</v>
+      </c>
+      <c r="G239" t="s">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="240" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A240" t="s">
+        <v>7</v>
+      </c>
+      <c r="B240" t="s">
+        <v>8</v>
+      </c>
+      <c r="C240" t="s">
+        <v>684</v>
+      </c>
+      <c r="E240" t="s">
+        <v>690</v>
+      </c>
+      <c r="G240" t="s">
+        <v>695</v>
+      </c>
+    </row>
+    <row r="241" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A241" t="s">
+        <v>7</v>
+      </c>
+      <c r="B241" t="s">
+        <v>8</v>
+      </c>
+      <c r="C241" t="s">
+        <v>696</v>
+      </c>
+      <c r="E241" t="s">
+        <v>698</v>
+      </c>
+      <c r="G241" t="s">
+        <v>697</v>
+      </c>
+    </row>
+    <row r="242" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A242" t="s">
+        <v>7</v>
+      </c>
+      <c r="B242" t="s">
+        <v>8</v>
+      </c>
+      <c r="C242" t="s">
+        <v>715</v>
+      </c>
+      <c r="E242" t="s">
+        <v>718</v>
+      </c>
+      <c r="G242" t="s">
+        <v>726</v>
+      </c>
+    </row>
+    <row r="243" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A243" t="s">
+        <v>7</v>
+      </c>
+      <c r="B243" t="s">
+        <v>8</v>
+      </c>
+      <c r="C243" t="s">
+        <v>716</v>
+      </c>
+      <c r="E243" t="s">
+        <v>719</v>
+      </c>
+      <c r="G243" t="s">
+        <v>727</v>
+      </c>
+    </row>
+    <row r="244" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A244" t="s">
+        <v>7</v>
+      </c>
+      <c r="B244" t="s">
+        <v>8</v>
+      </c>
+      <c r="C244" t="s">
+        <v>699</v>
+      </c>
+      <c r="E244" t="s">
+        <v>720</v>
+      </c>
+      <c r="G244" t="s">
+        <v>728</v>
+      </c>
+    </row>
+    <row r="245" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A245" t="s">
+        <v>7</v>
+      </c>
+      <c r="B245" t="s">
+        <v>8</v>
+      </c>
+      <c r="C245" t="s">
+        <v>700</v>
+      </c>
+      <c r="E245" t="s">
+        <v>721</v>
+      </c>
+      <c r="G245" t="s">
+        <v>710</v>
+      </c>
+    </row>
+    <row r="246" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A246" t="s">
+        <v>7</v>
+      </c>
+      <c r="B246" t="s">
+        <v>8</v>
+      </c>
+      <c r="C246" t="s">
+        <v>717</v>
+      </c>
+      <c r="E246" t="s">
+        <v>722</v>
+      </c>
+      <c r="G246" t="s">
+        <v>729</v>
+      </c>
+    </row>
+    <row r="247" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A247" t="s">
+        <v>7</v>
+      </c>
+      <c r="B247" t="s">
+        <v>8</v>
+      </c>
+      <c r="C247" t="s">
+        <v>701</v>
+      </c>
+      <c r="E247" t="s">
+        <v>723</v>
+      </c>
+      <c r="G247" t="s">
+        <v>730</v>
+      </c>
+    </row>
+    <row r="248" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A248" t="s">
+        <v>7</v>
+      </c>
+      <c r="B248" t="s">
+        <v>8</v>
+      </c>
+      <c r="C248" t="s">
+        <v>704</v>
+      </c>
+      <c r="E248" t="s">
+        <v>707</v>
+      </c>
+      <c r="G248" t="s">
+        <v>731</v>
+      </c>
+    </row>
+    <row r="249" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A249" t="s">
+        <v>7</v>
+      </c>
+      <c r="B249" t="s">
+        <v>8</v>
+      </c>
+      <c r="C249" t="s">
+        <v>705</v>
+      </c>
+      <c r="E249" t="s">
+        <v>708</v>
+      </c>
+      <c r="G249" t="s">
+        <v>713</v>
+      </c>
+    </row>
+    <row r="250" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A250" t="s">
+        <v>7</v>
+      </c>
+      <c r="B250" t="s">
+        <v>8</v>
+      </c>
+      <c r="C250" t="s">
+        <v>706</v>
+      </c>
+      <c r="E250" t="s">
+        <v>709</v>
+      </c>
+      <c r="G250" t="s">
+        <v>714</v>
+      </c>
+    </row>
+    <row r="251" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A251" t="s">
+        <v>7</v>
+      </c>
+      <c r="B251" t="s">
+        <v>8</v>
+      </c>
+      <c r="C251" t="s">
+        <v>702</v>
+      </c>
+      <c r="E251" t="s">
+        <v>724</v>
+      </c>
+      <c r="G251" t="s">
+        <v>711</v>
+      </c>
+    </row>
+    <row r="252" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A252" t="s">
+        <v>7</v>
+      </c>
+      <c r="B252" t="s">
+        <v>8</v>
+      </c>
+      <c r="C252" t="s">
+        <v>703</v>
+      </c>
+      <c r="E252" t="s">
+        <v>725</v>
+      </c>
+      <c r="G252" t="s">
+        <v>712</v>
       </c>
     </row>
   </sheetData>

</xml_diff>